<commit_message>
Add inventory management and equipment photos
</commit_message>
<xml_diff>
--- a/data/templates/NFC_Inventory_Import_Template.xlsx
+++ b/data/templates/NFC_Inventory_Import_Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="Rcda8e815ebc64c56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R32d7c49b4bbc466d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R03bec88663de4996"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="Rc505b70c00a549f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="Rb193db80559a469a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R7baea68a36c64486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R1c012ad657294ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R58c6d42c11ef4b52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="R9ab1bad1467641e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R96b6723f2dab4510"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,9 +404,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BundleContentsTable" displayName="BundleContentsTable" ref="A1:H4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H4"/>
-  <x:tableColumns count="8">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="BundleContentsTable" displayName="BundleContentsTable" ref="A1:I4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I4"/>
+  <x:tableColumns count="9">
     <x:tableColumn id="1" name="asset_code"/>
     <x:tableColumn id="2" name="component_name"/>
     <x:tableColumn id="3" name="manufacturer"/>
@@ -415,6 +415,7 @@
     <x:tableColumn id="6" name="quantity"/>
     <x:tableColumn id="7" name="required_on_return"/>
     <x:tableColumn id="8" name="notes"/>
+    <x:tableColumn id="9" name="photo_reference"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -806,8 +807,12 @@
       <x:c r="H12" s="58"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="63"/>
-      <x:c r="B13" s="62"/>
+      <x:c r="A13" s="63" t="str">
+        <x:v>Photos</x:v>
+      </x:c>
+      <x:c r="B13" s="62" t="str">
+        <x:v>Use a stable HTTPS image URL for each equipment row and bundle component. Keep the placeholder until a suitable photo is available.</x:v>
+      </x:c>
       <x:c r="C13" s="58"/>
       <x:c r="D13" s="58"/>
       <x:c r="E13" s="58"/>
@@ -998,7 +1003,9 @@
       <x:c r="S2" s="78" t="str"/>
       <x:c r="T2" s="78" t="str"/>
       <x:c r="U2" s="78" t="str"/>
-      <x:c r="V2" s="78" t="str"/>
+      <x:c r="V2" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="76" t="str">
@@ -1034,7 +1041,9 @@
       <x:c r="S3" s="78" t="str"/>
       <x:c r="T3" s="78" t="str"/>
       <x:c r="U3" s="78" t="str"/>
-      <x:c r="V3" s="78" t="str"/>
+      <x:c r="V3" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="76" t="str">
@@ -1070,7 +1079,9 @@
       <x:c r="S4" s="78" t="str"/>
       <x:c r="T4" s="78" t="str"/>
       <x:c r="U4" s="78" t="str"/>
-      <x:c r="V4" s="78" t="str"/>
+      <x:c r="V4" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="76" t="str">
@@ -1106,7 +1117,9 @@
       <x:c r="S5" s="78" t="str"/>
       <x:c r="T5" s="78" t="str"/>
       <x:c r="U5" s="78" t="str"/>
-      <x:c r="V5" s="78" t="str"/>
+      <x:c r="V5" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="76" t="str">
@@ -1142,7 +1155,9 @@
       <x:c r="S6" s="78" t="str"/>
       <x:c r="T6" s="78" t="str"/>
       <x:c r="U6" s="78" t="str"/>
-      <x:c r="V6" s="78" t="str"/>
+      <x:c r="V6" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="76" t="str">
@@ -1178,7 +1193,9 @@
       <x:c r="S7" s="78" t="str"/>
       <x:c r="T7" s="78" t="str"/>
       <x:c r="U7" s="78" t="str"/>
-      <x:c r="V7" s="78" t="str"/>
+      <x:c r="V7" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="76" t="str">
@@ -1214,7 +1231,9 @@
       <x:c r="S8" s="78" t="str"/>
       <x:c r="T8" s="78" t="str"/>
       <x:c r="U8" s="78" t="str"/>
-      <x:c r="V8" s="78" t="str"/>
+      <x:c r="V8" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="76" t="str">
@@ -1250,7 +1269,9 @@
       <x:c r="S9" s="78" t="str"/>
       <x:c r="T9" s="78" t="str"/>
       <x:c r="U9" s="78" t="str"/>
-      <x:c r="V9" s="78" t="str"/>
+      <x:c r="V9" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="76" t="str">
@@ -1286,7 +1307,9 @@
       <x:c r="S10" s="78" t="str"/>
       <x:c r="T10" s="78" t="str"/>
       <x:c r="U10" s="78" t="str"/>
-      <x:c r="V10" s="78" t="str"/>
+      <x:c r="V10" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="76" t="str">
@@ -1322,7 +1345,9 @@
       <x:c r="S11" s="78" t="str"/>
       <x:c r="T11" s="78" t="str"/>
       <x:c r="U11" s="78" t="str"/>
-      <x:c r="V11" s="78" t="str"/>
+      <x:c r="V11" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="76" t="str">
@@ -1358,7 +1383,9 @@
       <x:c r="S12" s="78" t="str"/>
       <x:c r="T12" s="78" t="str"/>
       <x:c r="U12" s="78" t="str"/>
-      <x:c r="V12" s="78" t="str"/>
+      <x:c r="V12" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="76" t="str">
@@ -1394,7 +1421,9 @@
       <x:c r="S13" s="78" t="str"/>
       <x:c r="T13" s="78" t="str"/>
       <x:c r="U13" s="78" t="str"/>
-      <x:c r="V13" s="78" t="str"/>
+      <x:c r="V13" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="76" t="str">
@@ -1430,7 +1459,9 @@
       <x:c r="S14" s="78" t="str"/>
       <x:c r="T14" s="78" t="str"/>
       <x:c r="U14" s="78" t="str"/>
-      <x:c r="V14" s="78" t="str"/>
+      <x:c r="V14" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="76" t="str">
@@ -1466,7 +1497,9 @@
       <x:c r="S15" s="78" t="str"/>
       <x:c r="T15" s="78" t="str"/>
       <x:c r="U15" s="78" t="str"/>
-      <x:c r="V15" s="78" t="str"/>
+      <x:c r="V15" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="76" t="str">
@@ -1502,7 +1535,9 @@
       <x:c r="S16" s="78" t="str"/>
       <x:c r="T16" s="78" t="str"/>
       <x:c r="U16" s="78" t="str"/>
-      <x:c r="V16" s="78" t="str"/>
+      <x:c r="V16" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="76" t="str">
@@ -1538,7 +1573,9 @@
       <x:c r="S17" s="78" t="str"/>
       <x:c r="T17" s="78" t="str"/>
       <x:c r="U17" s="78" t="str"/>
-      <x:c r="V17" s="78" t="str"/>
+      <x:c r="V17" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="76" t="str">
@@ -1574,7 +1611,9 @@
       <x:c r="S18" s="78" t="str"/>
       <x:c r="T18" s="78" t="str"/>
       <x:c r="U18" s="78" t="str"/>
-      <x:c r="V18" s="78" t="str"/>
+      <x:c r="V18" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="76" t="str">
@@ -1610,7 +1649,9 @@
       <x:c r="S19" s="78" t="str"/>
       <x:c r="T19" s="78" t="str"/>
       <x:c r="U19" s="78" t="str"/>
-      <x:c r="V19" s="78" t="str"/>
+      <x:c r="V19" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="76" t="str">
@@ -1646,7 +1687,9 @@
       <x:c r="S20" s="78" t="str"/>
       <x:c r="T20" s="78" t="str"/>
       <x:c r="U20" s="78" t="str"/>
-      <x:c r="V20" s="78" t="str"/>
+      <x:c r="V20" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="76" t="str">
@@ -1682,7 +1725,9 @@
       <x:c r="S21" s="78" t="str"/>
       <x:c r="T21" s="78" t="str"/>
       <x:c r="U21" s="78" t="str"/>
-      <x:c r="V21" s="78" t="str"/>
+      <x:c r="V21" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="76" t="str">
@@ -1718,7 +1763,9 @@
       <x:c r="S22" s="78" t="str"/>
       <x:c r="T22" s="78" t="str"/>
       <x:c r="U22" s="78" t="str"/>
-      <x:c r="V22" s="78" t="str"/>
+      <x:c r="V22" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="76" t="str">
@@ -1754,7 +1801,9 @@
       <x:c r="S23" s="78" t="str"/>
       <x:c r="T23" s="78" t="str"/>
       <x:c r="U23" s="78" t="str"/>
-      <x:c r="V23" s="78" t="str"/>
+      <x:c r="V23" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="76" t="str">
@@ -1790,7 +1839,9 @@
       <x:c r="S24" s="78" t="str"/>
       <x:c r="T24" s="78" t="str"/>
       <x:c r="U24" s="78" t="str"/>
-      <x:c r="V24" s="78" t="str"/>
+      <x:c r="V24" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="76" t="str">
@@ -1826,7 +1877,9 @@
       <x:c r="S25" s="78" t="str"/>
       <x:c r="T25" s="78" t="str"/>
       <x:c r="U25" s="78" t="str"/>
-      <x:c r="V25" s="78" t="str"/>
+      <x:c r="V25" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="76" t="str">
@@ -1862,7 +1915,9 @@
       <x:c r="S26" s="78" t="str"/>
       <x:c r="T26" s="78" t="str"/>
       <x:c r="U26" s="78" t="str"/>
-      <x:c r="V26" s="78" t="str"/>
+      <x:c r="V26" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="76" t="str">
@@ -1898,7 +1953,9 @@
       <x:c r="S27" s="78" t="str"/>
       <x:c r="T27" s="78" t="str"/>
       <x:c r="U27" s="78" t="str"/>
-      <x:c r="V27" s="78" t="str"/>
+      <x:c r="V27" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="76" t="str">
@@ -1934,7 +1991,9 @@
       <x:c r="S28" s="78" t="str"/>
       <x:c r="T28" s="78" t="str"/>
       <x:c r="U28" s="78" t="str"/>
-      <x:c r="V28" s="78" t="str"/>
+      <x:c r="V28" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="76" t="str">
@@ -1970,7 +2029,9 @@
       <x:c r="S29" s="78" t="str"/>
       <x:c r="T29" s="78" t="str"/>
       <x:c r="U29" s="78" t="str"/>
-      <x:c r="V29" s="78" t="str"/>
+      <x:c r="V29" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="76" t="str">
@@ -2006,7 +2067,9 @@
       <x:c r="S30" s="78" t="str"/>
       <x:c r="T30" s="78" t="str"/>
       <x:c r="U30" s="78" t="str"/>
-      <x:c r="V30" s="78" t="str"/>
+      <x:c r="V30" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="76" t="str">
@@ -2042,7 +2105,9 @@
       <x:c r="S31" s="78" t="str"/>
       <x:c r="T31" s="78" t="str"/>
       <x:c r="U31" s="78" t="str"/>
-      <x:c r="V31" s="78" t="str"/>
+      <x:c r="V31" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="76" t="str">
@@ -2078,7 +2143,9 @@
       <x:c r="S32" s="78" t="str"/>
       <x:c r="T32" s="78" t="str"/>
       <x:c r="U32" s="78" t="str"/>
-      <x:c r="V32" s="78" t="str"/>
+      <x:c r="V32" s="78" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="5">
@@ -2100,7 +2167,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4ba3e61930f4410"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R383badd084114f43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2120,6 +2187,7 @@
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -2147,6 +2215,9 @@
       <x:c r="H1" s="38" t="str">
         <x:v>notes</x:v>
       </x:c>
+      <x:c r="I1" t="str">
+        <x:v>photo_reference</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="77" t="str">
@@ -2165,6 +2236,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H2" s="78" t="str"/>
+      <x:c r="I2" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="77" t="str">
@@ -2183,6 +2257,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H3" s="78" t="str"/>
+      <x:c r="I3" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="77" t="str">
@@ -2201,6 +2278,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H4" s="78" t="str"/>
+      <x:c r="I4" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
@@ -2216,7 +2296,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd29ceefbe4cb473e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdec5bddf0d4e455a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2328,7 +2408,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52629735925644c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4793a36a75324730"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2458,7 +2538,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42f40225afcb4aae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd23e6904df6e47d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix theme toggle and add equipment photos
</commit_message>
<xml_diff>
--- a/data/templates/NFC_Inventory_Import_Template.xlsx
+++ b/data/templates/NFC_Inventory_Import_Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R7baea68a36c64486"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R1c012ad657294ffc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R58c6d42c11ef4b52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="R9ab1bad1467641e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R96b6723f2dab4510"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R27ae6c101c524cea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="Rd70638f0cb154ec8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R6db5d35c805a4367"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="R309d68c952674a0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R8918985fc9914dad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,7 +811,7 @@
         <x:v>Photos</x:v>
       </x:c>
       <x:c r="B13" s="62" t="str">
-        <x:v>Use a stable HTTPS image URL for each equipment row and bundle component. Keep the placeholder until a suitable photo is available.</x:v>
+        <x:v>Use a stable HTTPS image URL for each equipment row and bundle component. Product reference images are listed in docs/image-sources.md; replace them with lab-owned photos when available. Keep the placeholder when the exact model is unknown.</x:v>
       </x:c>
       <x:c r="C13" s="58"/>
       <x:c r="D13" s="58"/>
@@ -1004,7 +1004,7 @@
       <x:c r="T2" s="78" t="str"/>
       <x:c r="U2" s="78" t="str"/>
       <x:c r="V2" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/misty-ii.png</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1042,7 +1042,7 @@
       <x:c r="T3" s="78" t="str"/>
       <x:c r="U3" s="78" t="str"/>
       <x:c r="V3" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/misty-ii.png</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1080,7 +1080,7 @@
       <x:c r="T4" s="78" t="str"/>
       <x:c r="U4" s="78" t="str"/>
       <x:c r="V4" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-wireless.png</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1118,7 +1118,7 @@
       <x:c r="T5" s="78" t="str"/>
       <x:c r="U5" s="78" t="str"/>
       <x:c r="V5" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-lite.png</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1308,7 +1308,7 @@
       <x:c r="T10" s="78" t="str"/>
       <x:c r="U10" s="78" t="str"/>
       <x:c r="V10" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/azure-kinect-dk.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1346,7 +1346,7 @@
       <x:c r="T11" s="78" t="str"/>
       <x:c r="U11" s="78" t="str"/>
       <x:c r="V11" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/azure-kinect-dk.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1384,7 +1384,7 @@
       <x:c r="T12" s="78" t="str"/>
       <x:c r="U12" s="78" t="str"/>
       <x:c r="V12" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/anker-powerconf-c200.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1422,7 +1422,7 @@
       <x:c r="T13" s="78" t="str"/>
       <x:c r="U13" s="78" t="str"/>
       <x:c r="V13" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/anker-powerconf-c200.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1460,7 +1460,7 @@
       <x:c r="T14" s="78" t="str"/>
       <x:c r="U14" s="78" t="str"/>
       <x:c r="V14" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/victiv-tripod.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1498,7 +1498,7 @@
       <x:c r="T15" s="78" t="str"/>
       <x:c r="U15" s="78" t="str"/>
       <x:c r="V15" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/victiv-tripod.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1536,7 +1536,7 @@
       <x:c r="T16" s="78" t="str"/>
       <x:c r="U16" s="78" t="str"/>
       <x:c r="V16" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/victiv-tripod.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1650,7 +1650,7 @@
       <x:c r="T19" s="78" t="str"/>
       <x:c r="U19" s="78" t="str"/>
       <x:c r="V19" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/lammcou-small-tripod.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1688,7 +1688,7 @@
       <x:c r="T20" s="78" t="str"/>
       <x:c r="U20" s="78" t="str"/>
       <x:c r="V20" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/lammcou-small-tripod.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1878,7 +1878,7 @@
       <x:c r="T25" s="78" t="str"/>
       <x:c r="U25" s="78" t="str"/>
       <x:c r="V25" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/boya-v30.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1916,7 +1916,7 @@
       <x:c r="T26" s="78" t="str"/>
       <x:c r="U26" s="78" t="str"/>
       <x:c r="V26" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/dji-mic-mini.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2030,7 +2030,7 @@
       <x:c r="T29" s="78" t="str"/>
       <x:c r="U29" s="78" t="str"/>
       <x:c r="V29" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/belkin-bsv804.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2068,7 +2068,7 @@
       <x:c r="T30" s="78" t="str"/>
       <x:c r="U30" s="78" t="str"/>
       <x:c r="V30" s="78" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/tapo-p110.jpg</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2167,7 +2167,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R383badd084114f43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1e1e7b7b4224b5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2237,7 +2237,7 @@
       </x:c>
       <x:c r="H2" s="78" t="str"/>
       <x:c r="I2" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-wireless.png</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2296,7 +2296,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdec5bddf0d4e455a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf447d4fd9bc14bbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2408,7 +2408,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4793a36a75324730"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17535bd80f314851"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2538,7 +2538,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd23e6904df6e47d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f3a24519bad4cdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Identify Lenovo Tab M10 models
</commit_message>
<xml_diff>
--- a/data/templates/NFC_Inventory_Import_Template.xlsx
+++ b/data/templates/NFC_Inventory_Import_Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R6a93ed6a73084ced"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R02bb2c5185b44264"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R07f74c1e96a24817"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="R47d29cfc2359400a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="Rc9732e0284f84455"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R07fea3f966bf445e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R4035cf9c9ed2443b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R36221e72967543d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="R1f1ec372e0984d85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R50412a6762a143ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -219,9 +219,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TAB-001</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Lenovo Tab M10</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Tablets</x:t>
@@ -1797,19 +1794,25 @@
       <x:c r="A8" s="9" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="B8" s="10" t="s">
+      <x:c r="B8" s="10" t="str">
+        <x:v>Lenovo Tab M10 (3rd Gen)</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C8" s="10" t="s">
-        <x:v>70</x:v>
-      </x:c>
       <x:c r="D8" s="10" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="E8" s="4"/>
-      <x:c r="F8" s="4"/>
+      <x:c r="E8" s="4" t="str">
+        <x:v>Lenovo</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>TB328FU</x:v>
+      </x:c>
       <x:c r="G8" s="4"/>
-      <x:c r="H8" s="11"/>
+      <x:c r="H8" s="11" t="str">
+        <x:v>3rd Gen</x:v>
+      </x:c>
       <x:c r="I8" s="11"/>
       <x:c r="J8" s="11"/>
       <x:c r="K8" s="12" t="s">
@@ -1828,26 +1831,32 @@
       <x:c r="T8" s="11"/>
       <x:c r="U8" s="11"/>
       <x:c r="V8" s="11" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="37.5">
       <x:c r="A9" s="9" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="B9" s="10" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B9" s="10" t="str">
+        <x:v>Lenovo Tab M10 (3rd Gen)</x:v>
+      </x:c>
+      <x:c r="C9" s="10" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C9" s="10" t="s">
-        <x:v>70</x:v>
-      </x:c>
       <x:c r="D9" s="10" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="E9" s="4"/>
-      <x:c r="F9" s="4"/>
+      <x:c r="E9" s="4" t="str">
+        <x:v>Lenovo</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>TB328FU</x:v>
+      </x:c>
       <x:c r="G9" s="4"/>
-      <x:c r="H9" s="11"/>
+      <x:c r="H9" s="11" t="str">
+        <x:v>3rd Gen</x:v>
+      </x:c>
       <x:c r="I9" s="11"/>
       <x:c r="J9" s="11"/>
       <x:c r="K9" s="12" t="s">
@@ -1866,18 +1875,18 @@
       <x:c r="T9" s="11"/>
       <x:c r="U9" s="11"/>
       <x:c r="V9" s="11" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="37.5">
       <x:c r="A10" s="9" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="B10" s="10" t="s">
+      <x:c r="C10" s="10" t="s">
         <x:v>74</x:v>
-      </x:c>
-      <x:c r="C10" s="10" t="s">
-        <x:v>75</x:v>
       </x:c>
       <x:c r="D10" s="10" t="s">
         <x:v>51</x:v>
@@ -1904,18 +1913,18 @@
       <x:c r="T10" s="11"/>
       <x:c r="U10" s="11"/>
       <x:c r="V10" s="11" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="37.5">
       <x:c r="A11" s="9" t="s">
-        <x:v>76</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="B11" s="10" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="s">
         <x:v>74</x:v>
-      </x:c>
-      <x:c r="C11" s="10" t="s">
-        <x:v>75</x:v>
       </x:c>
       <x:c r="D11" s="10" t="s">
         <x:v>51</x:v>
@@ -1942,15 +1951,15 @@
       <x:c r="T11" s="11"/>
       <x:c r="U11" s="11"/>
       <x:c r="V11" s="11" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="37.5">
       <x:c r="A12" s="9" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="s">
         <x:v>77</x:v>
-      </x:c>
-      <x:c r="B12" s="10" t="s">
-        <x:v>78</x:v>
       </x:c>
       <x:c r="C12" s="10" t="str">
         <x:v>Cameras</x:v>
@@ -1980,15 +1989,15 @@
       <x:c r="T12" s="11"/>
       <x:c r="U12" s="11"/>
       <x:c r="V12" s="11" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="37.5">
       <x:c r="A13" s="9" t="s">
-        <x:v>80</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B13" s="10" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C13" s="10" t="str">
         <x:v>Cameras</x:v>
@@ -2018,15 +2027,15 @@
       <x:c r="T13" s="11"/>
       <x:c r="U13" s="11"/>
       <x:c r="V13" s="11" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="37.5">
       <x:c r="A14" s="9" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="B14" s="10" t="s">
         <x:v>81</x:v>
-      </x:c>
-      <x:c r="B14" s="10" t="s">
-        <x:v>82</x:v>
       </x:c>
       <x:c r="C14" s="10" t="str">
         <x:v>Cameras</x:v>
@@ -2035,14 +2044,14 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="E14" s="4" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="s">
         <x:v>83</x:v>
-      </x:c>
-      <x:c r="F14" s="4" t="s">
-        <x:v>84</x:v>
       </x:c>
       <x:c r="G14" s="4"/>
       <x:c r="H14" s="11" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="I14" s="11"/>
       <x:c r="J14" s="11"/>
@@ -2063,18 +2072,18 @@
       <x:c r="S14" s="11"/>
       <x:c r="T14" s="11"/>
       <x:c r="U14" s="11" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="V14" s="11" t="s">
         <x:v>86</x:v>
-      </x:c>
-      <x:c r="V14" s="11" t="s">
-        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="37.5">
       <x:c r="A15" s="9" t="s">
-        <x:v>88</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B15" s="10" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C15" s="10" t="str">
         <x:v>Cameras</x:v>
@@ -2083,14 +2092,14 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="E15" s="4" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="s">
         <x:v>83</x:v>
-      </x:c>
-      <x:c r="F15" s="4" t="s">
-        <x:v>84</x:v>
       </x:c>
       <x:c r="G15" s="4"/>
       <x:c r="H15" s="11" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="I15" s="11"/>
       <x:c r="J15" s="11"/>
@@ -2111,21 +2120,21 @@
       <x:c r="S15" s="11"/>
       <x:c r="T15" s="11"/>
       <x:c r="U15" s="11" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="V15" s="11" t="s">
         <x:v>86</x:v>
-      </x:c>
-      <x:c r="V15" s="11" t="s">
-        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="37.5">
       <x:c r="A16" s="9" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="s">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="B16" s="10" t="s">
-        <x:v>90</x:v>
-      </x:c>
       <x:c r="C16" s="10" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D16" s="10" t="s">
         <x:v>51</x:v>
@@ -2152,18 +2161,18 @@
       <x:c r="T16" s="11"/>
       <x:c r="U16" s="11"/>
       <x:c r="V16" s="11" t="s">
-        <x:v>91</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="37.5">
       <x:c r="A17" s="9" t="s">
-        <x:v>92</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B17" s="10" t="s">
-        <x:v>90</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C17" s="10" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D17" s="10" t="s">
         <x:v>51</x:v>
@@ -2190,18 +2199,18 @@
       <x:c r="T17" s="11"/>
       <x:c r="U17" s="11"/>
       <x:c r="V17" s="11" t="s">
-        <x:v>91</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="37.5">
       <x:c r="A18" s="9" t="s">
-        <x:v>93</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B18" s="10" t="s">
-        <x:v>90</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C18" s="10" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D18" s="10" t="s">
         <x:v>51</x:v>
@@ -2228,18 +2237,18 @@
       <x:c r="T18" s="11"/>
       <x:c r="U18" s="11"/>
       <x:c r="V18" s="11" t="s">
-        <x:v>91</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="37.5">
       <x:c r="A19" s="9" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="s">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="B19" s="10" t="s">
-        <x:v>95</x:v>
-      </x:c>
       <x:c r="C19" s="10" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D19" s="10" t="s">
         <x:v>51</x:v>
@@ -2266,18 +2275,18 @@
       <x:c r="T19" s="11"/>
       <x:c r="U19" s="11"/>
       <x:c r="V19" s="11" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="37.5">
       <x:c r="A20" s="9" t="s">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B20" s="10" t="s">
-        <x:v>95</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C20" s="10" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D20" s="10" t="s">
         <x:v>51</x:v>
@@ -2304,18 +2313,18 @@
       <x:c r="T20" s="11"/>
       <x:c r="U20" s="11"/>
       <x:c r="V20" s="11" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="37.5">
       <x:c r="A21" s="9" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="B21" s="10" t="s">
-        <x:v>98</x:v>
-      </x:c>
       <x:c r="C21" s="10" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D21" s="10" t="s">
         <x:v>51</x:v>
@@ -2342,18 +2351,18 @@
       <x:c r="T21" s="11"/>
       <x:c r="U21" s="11"/>
       <x:c r="V21" s="11" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="37.5">
       <x:c r="A22" s="9" t="s">
-        <x:v>100</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B22" s="10" t="s">
-        <x:v>98</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C22" s="10" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D22" s="10" t="s">
         <x:v>51</x:v>
@@ -2380,18 +2389,18 @@
       <x:c r="T22" s="11"/>
       <x:c r="U22" s="11"/>
       <x:c r="V22" s="11" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="37.5">
       <x:c r="A23" s="9" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="B23" s="10" t="s">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="B23" s="10" t="s">
-        <x:v>102</x:v>
-      </x:c>
       <x:c r="C23" s="10" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D23" s="10" t="s">
         <x:v>51</x:v>
@@ -2418,18 +2427,18 @@
       <x:c r="T23" s="11"/>
       <x:c r="U23" s="11"/>
       <x:c r="V23" s="11" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="37.5">
       <x:c r="A24" s="9" t="s">
-        <x:v>103</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B24" s="10" t="s">
-        <x:v>102</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C24" s="10" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D24" s="10" t="s">
         <x:v>51</x:v>
@@ -2456,31 +2465,31 @@
       <x:c r="T24" s="11"/>
       <x:c r="U24" s="11"/>
       <x:c r="V24" s="11" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="37.5">
       <x:c r="A25" s="9" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="B25" s="10" t="s">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="B25" s="10" t="s">
+      <x:c r="C25" s="10" t="s">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="C25" s="10" t="s">
+      <x:c r="D25" s="10" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E25" s="4" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="D25" s="10" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E25" s="4" t="s">
+      <x:c r="F25" s="4" t="s">
         <x:v>107</x:v>
-      </x:c>
-      <x:c r="F25" s="4" t="s">
-        <x:v>108</x:v>
       </x:c>
       <x:c r="G25" s="4"/>
       <x:c r="H25" s="11" t="s">
-        <x:v>109</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="I25" s="11"/>
       <x:c r="J25" s="11"/>
@@ -2500,31 +2509,31 @@
       <x:c r="T25" s="11"/>
       <x:c r="U25" s="11"/>
       <x:c r="V25" s="11" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="37.5">
       <x:c r="A26" s="9" t="s">
-        <x:v>111</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B26" s="10" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="C26" s="10" t="s">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="C26" s="10" t="s">
+      <x:c r="D26" s="10" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E26" s="4" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="D26" s="10" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E26" s="4" t="s">
+      <x:c r="F26" s="4" t="s">
         <x:v>107</x:v>
-      </x:c>
-      <x:c r="F26" s="4" t="s">
-        <x:v>108</x:v>
       </x:c>
       <x:c r="G26" s="4"/>
       <x:c r="H26" s="11" t="s">
-        <x:v>109</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="I26" s="11"/>
       <x:c r="J26" s="11"/>
@@ -2544,31 +2553,31 @@
       <x:c r="T26" s="11"/>
       <x:c r="U26" s="11"/>
       <x:c r="V26" s="11" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="37.5">
       <x:c r="A27" s="9" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="B27" s="10" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="B27" s="10" t="s">
+      <x:c r="C27" s="10" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="C27" s="10" t="s">
+      <x:c r="D27" s="10" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E27" s="4" t="s">
         <x:v>114</x:v>
       </x:c>
-      <x:c r="D27" s="10" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E27" s="4" t="s">
+      <x:c r="F27" s="4" t="s">
         <x:v>115</x:v>
-      </x:c>
-      <x:c r="F27" s="4" t="s">
-        <x:v>116</x:v>
       </x:c>
       <x:c r="G27" s="4"/>
       <x:c r="H27" s="11" t="s">
-        <x:v>117</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="I27" s="11"/>
       <x:c r="J27" s="11"/>
@@ -2588,18 +2597,18 @@
       <x:c r="T27" s="11"/>
       <x:c r="U27" s="11"/>
       <x:c r="V27" s="11" t="s">
-        <x:v>118</x:v>
+        <x:v>117</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="37.5">
       <x:c r="A28" s="9" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="B28" s="10" t="s">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="B28" s="10" t="s">
-        <x:v>120</x:v>
-      </x:c>
       <x:c r="C28" s="10" t="s">
-        <x:v>114</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="D28" s="10" t="s">
         <x:v>51</x:v>
@@ -2626,18 +2635,18 @@
       <x:c r="T28" s="11"/>
       <x:c r="U28" s="11"/>
       <x:c r="V28" s="11" t="s">
-        <x:v>121</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="37.5">
       <x:c r="A29" s="9" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="B29" s="10" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="B29" s="10" t="s">
+      <x:c r="C29" s="10" t="s">
         <x:v>123</x:v>
-      </x:c>
-      <x:c r="C29" s="10" t="s">
-        <x:v>124</x:v>
       </x:c>
       <x:c r="D29" s="10" t="s">
         <x:v>51</x:v>
@@ -2664,18 +2673,18 @@
       <x:c r="T29" s="11"/>
       <x:c r="U29" s="11"/>
       <x:c r="V29" s="11" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="37.5">
       <x:c r="A30" s="9" t="s">
-        <x:v>125</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B30" s="10" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="C30" s="10" t="s">
         <x:v>123</x:v>
-      </x:c>
-      <x:c r="C30" s="10" t="s">
-        <x:v>124</x:v>
       </x:c>
       <x:c r="D30" s="10" t="s">
         <x:v>51</x:v>
@@ -2702,18 +2711,18 @@
       <x:c r="T30" s="11"/>
       <x:c r="U30" s="11"/>
       <x:c r="V30" s="11" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="37.5">
       <x:c r="A31" s="9" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="B31" s="10" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="B31" s="10" t="s">
-        <x:v>127</x:v>
-      </x:c>
       <x:c r="C31" s="10" t="s">
-        <x:v>124</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="D31" s="10" t="s">
         <x:v>51</x:v>
@@ -2740,18 +2749,18 @@
       <x:c r="T31" s="11"/>
       <x:c r="U31" s="11"/>
       <x:c r="V31" s="11" t="s">
-        <x:v>128</x:v>
+        <x:v>127</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="37.5">
       <x:c r="A32" s="9" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="B32" s="10" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="B32" s="10" t="s">
-        <x:v>130</x:v>
-      </x:c>
       <x:c r="C32" s="10" t="s">
-        <x:v>124</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="D32" s="10" t="s">
         <x:v>51</x:v>
@@ -2778,31 +2787,31 @@
       <x:c r="T32" s="11"/>
       <x:c r="U32" s="11"/>
       <x:c r="V32" s="11" t="s">
-        <x:v>131</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="87.5">
       <x:c r="A33" s="9" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="B33" s="10" t="s">
         <x:v>132</x:v>
       </x:c>
-      <x:c r="B33" s="10" t="s">
+      <x:c r="C33" s="10" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="C33" s="10" t="s">
+      <x:c r="D33" s="10" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E33" s="4" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="D33" s="10" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E33" s="4" t="s">
+      <x:c r="F33" s="4" t="s">
         <x:v>135</x:v>
-      </x:c>
-      <x:c r="F33" s="4" t="s">
-        <x:v>136</x:v>
       </x:c>
       <x:c r="G33" s="4"/>
       <x:c r="H33" s="11" t="s">
-        <x:v>137</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="I33" s="11"/>
       <x:c r="J33" s="11"/>
@@ -2823,34 +2832,34 @@
       <x:c r="S33" s="11"/>
       <x:c r="T33" s="11"/>
       <x:c r="U33" s="11" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="V33" s="11" t="s">
         <x:v>138</x:v>
-      </x:c>
-      <x:c r="V33" s="11" t="s">
-        <x:v>139</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="87.5">
       <x:c r="A34" s="9" t="s">
-        <x:v>140</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B34" s="10" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="C34" s="10" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="C34" s="10" t="s">
+      <x:c r="D34" s="10" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E34" s="4" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="D34" s="10" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E34" s="4" t="s">
+      <x:c r="F34" s="4" t="s">
         <x:v>135</x:v>
-      </x:c>
-      <x:c r="F34" s="4" t="s">
-        <x:v>136</x:v>
       </x:c>
       <x:c r="G34" s="4"/>
       <x:c r="H34" s="11" t="s">
-        <x:v>137</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="I34" s="11"/>
       <x:c r="J34" s="11"/>
@@ -2871,18 +2880,18 @@
       <x:c r="S34" s="11"/>
       <x:c r="T34" s="11"/>
       <x:c r="U34" s="11" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="V34" s="11" t="s">
         <x:v>138</x:v>
-      </x:c>
-      <x:c r="V34" s="11" t="s">
-        <x:v>139</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="B35" t="s">
         <x:v>141</x:v>
-      </x:c>
-      <x:c r="B35" t="s">
-        <x:v>142</x:v>
       </x:c>
       <x:c r="C35" t="str">
         <x:v>Cameras</x:v>
@@ -2891,13 +2900,13 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="E35" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="F35" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="F35" t="s">
+      <x:c r="H35" t="s">
         <x:v>144</x:v>
-      </x:c>
-      <x:c r="H35" t="s">
-        <x:v>145</x:v>
       </x:c>
       <x:c r="K35" t="s">
         <x:v>52</x:v>
@@ -2909,18 +2918,18 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U35" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="V35" t="s">
         <x:v>146</x:v>
-      </x:c>
-      <x:c r="V35" t="s">
-        <x:v>147</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="B36" t="s">
         <x:v>148</x:v>
-      </x:c>
-      <x:c r="B36" t="s">
-        <x:v>149</x:v>
       </x:c>
       <x:c r="C36" t="str">
         <x:v>Cameras</x:v>
@@ -2929,13 +2938,13 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="E36" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="F36" t="s">
         <x:v>150</x:v>
       </x:c>
-      <x:c r="F36" t="s">
+      <x:c r="H36" t="s">
         <x:v>151</x:v>
-      </x:c>
-      <x:c r="H36" t="s">
-        <x:v>152</x:v>
       </x:c>
       <x:c r="K36" t="s">
         <x:v>52</x:v>
@@ -2947,33 +2956,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U36" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="V36" t="s">
         <x:v>153</x:v>
-      </x:c>
-      <x:c r="V36" t="s">
-        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="B37" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="B37" t="s">
+      <x:c r="C37" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D37" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E37" t="s">
         <x:v>156</x:v>
       </x:c>
-      <x:c r="C37" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="D37" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E37" t="s">
+      <x:c r="F37" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="F37" t="s">
+      <x:c r="H37" t="s">
         <x:v>158</x:v>
-      </x:c>
-      <x:c r="H37" t="s">
-        <x:v>159</x:v>
       </x:c>
       <x:c r="K37" t="s">
         <x:v>52</x:v>
@@ -2985,33 +2994,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U37" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="V37" t="s">
         <x:v>160</x:v>
-      </x:c>
-      <x:c r="V37" t="s">
-        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="s">
-        <x:v>162</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B38" t="s">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="C38" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D38" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E38" t="s">
         <x:v>156</x:v>
       </x:c>
-      <x:c r="C38" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="D38" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E38" t="s">
+      <x:c r="F38" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="F38" t="s">
+      <x:c r="H38" t="s">
         <x:v>158</x:v>
-      </x:c>
-      <x:c r="H38" t="s">
-        <x:v>159</x:v>
       </x:c>
       <x:c r="K38" t="s">
         <x:v>52</x:v>
@@ -3023,33 +3032,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U38" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="V38" t="s">
         <x:v>160</x:v>
-      </x:c>
-      <x:c r="V38" t="s">
-        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="B39" t="s">
         <x:v>163</x:v>
       </x:c>
-      <x:c r="B39" t="s">
+      <x:c r="C39" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D39" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E39" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="F39" t="s">
         <x:v>164</x:v>
       </x:c>
-      <x:c r="C39" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="D39" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E39" t="s">
-        <x:v>157</x:v>
-      </x:c>
-      <x:c r="F39" t="s">
+      <x:c r="H39" t="s">
         <x:v>165</x:v>
-      </x:c>
-      <x:c r="H39" t="s">
-        <x:v>166</x:v>
       </x:c>
       <x:c r="K39" t="s">
         <x:v>52</x:v>
@@ -3061,30 +3070,30 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U39" t="s">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="V39" t="s">
         <x:v>167</x:v>
-      </x:c>
-      <x:c r="V39" t="s">
-        <x:v>168</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="B40" t="s">
         <x:v>169</x:v>
       </x:c>
-      <x:c r="B40" t="s">
+      <x:c r="C40" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="D40" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="F40" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="C40" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="D40" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="F40" t="s">
+      <x:c r="H40" t="s">
         <x:v>171</x:v>
-      </x:c>
-      <x:c r="H40" t="s">
-        <x:v>172</x:v>
       </x:c>
       <x:c r="K40" t="s">
         <x:v>52</x:v>
@@ -3096,33 +3105,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U40" t="s">
-        <x:v>173</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="V40" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" t="s">
-        <x:v>174</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B41" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="C41" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="C41" t="s">
+      <x:c r="D41" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E41" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="D41" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E41" t="s">
+      <x:c r="F41" t="s">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="F41" t="s">
+      <x:c r="H41" t="s">
         <x:v>136</x:v>
-      </x:c>
-      <x:c r="H41" t="s">
-        <x:v>137</x:v>
       </x:c>
       <x:c r="K41" t="s">
         <x:v>52</x:v>
@@ -3134,33 +3143,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U41" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="V41" t="s">
         <x:v>138</x:v>
-      </x:c>
-      <x:c r="V41" t="s">
-        <x:v>139</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="B42" t="s">
         <x:v>175</x:v>
       </x:c>
-      <x:c r="B42" t="s">
+      <x:c r="C42" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="D42" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E42" t="s">
         <x:v>176</x:v>
       </x:c>
-      <x:c r="C42" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="D42" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E42" t="s">
+      <x:c r="F42" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="F42" t="s">
+      <x:c r="H42" t="s">
         <x:v>178</x:v>
-      </x:c>
-      <x:c r="H42" t="s">
-        <x:v>179</x:v>
       </x:c>
       <x:c r="K42" t="s">
         <x:v>52</x:v>
@@ -3172,33 +3181,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U42" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="V42" t="s">
         <x:v>180</x:v>
-      </x:c>
-      <x:c r="V42" t="s">
-        <x:v>181</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" t="s">
-        <x:v>182</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="B43" t="s">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="C43" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="D43" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E43" t="s">
         <x:v>176</x:v>
       </x:c>
-      <x:c r="C43" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="D43" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E43" t="s">
+      <x:c r="F43" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="F43" t="s">
+      <x:c r="H43" t="s">
         <x:v>178</x:v>
-      </x:c>
-      <x:c r="H43" t="s">
-        <x:v>179</x:v>
       </x:c>
       <x:c r="K43" t="s">
         <x:v>52</x:v>
@@ -3210,33 +3219,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U43" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="V43" t="s">
         <x:v>180</x:v>
-      </x:c>
-      <x:c r="V43" t="s">
-        <x:v>181</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" t="s">
-        <x:v>183</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="B44" t="s">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="C44" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="D44" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E44" t="s">
         <x:v>176</x:v>
       </x:c>
-      <x:c r="C44" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="D44" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E44" t="s">
+      <x:c r="F44" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="F44" t="s">
+      <x:c r="H44" t="s">
         <x:v>178</x:v>
-      </x:c>
-      <x:c r="H44" t="s">
-        <x:v>179</x:v>
       </x:c>
       <x:c r="K44" t="s">
         <x:v>52</x:v>
@@ -3248,33 +3257,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U44" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="V44" t="s">
         <x:v>180</x:v>
-      </x:c>
-      <x:c r="V44" t="s">
-        <x:v>181</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" t="s">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="B45" t="s">
         <x:v>184</x:v>
       </x:c>
-      <x:c r="B45" t="s">
+      <x:c r="C45" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="D45" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E45" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="C45" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="D45" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E45" t="s">
+      <x:c r="F45" t="s">
         <x:v>186</x:v>
       </x:c>
-      <x:c r="F45" t="s">
+      <x:c r="H45" t="s">
         <x:v>187</x:v>
-      </x:c>
-      <x:c r="H45" t="s">
-        <x:v>188</x:v>
       </x:c>
       <x:c r="K45" t="s">
         <x:v>52</x:v>
@@ -3286,33 +3295,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U45" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="V45" t="s">
         <x:v>189</x:v>
-      </x:c>
-      <x:c r="V45" t="s">
-        <x:v>190</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" t="s">
-        <x:v>191</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B46" t="s">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="C46" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="D46" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E46" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="C46" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="D46" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E46" t="s">
+      <x:c r="F46" t="s">
         <x:v>186</x:v>
       </x:c>
-      <x:c r="F46" t="s">
+      <x:c r="H46" t="s">
         <x:v>187</x:v>
-      </x:c>
-      <x:c r="H46" t="s">
-        <x:v>188</x:v>
       </x:c>
       <x:c r="K46" t="s">
         <x:v>52</x:v>
@@ -3324,33 +3333,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U46" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="V46" t="s">
         <x:v>189</x:v>
-      </x:c>
-      <x:c r="V46" t="s">
-        <x:v>190</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" t="s">
-        <x:v>192</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="B47" t="s">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="C47" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="D47" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E47" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="C47" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="D47" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E47" t="s">
+      <x:c r="F47" t="s">
         <x:v>186</x:v>
       </x:c>
-      <x:c r="F47" t="s">
+      <x:c r="H47" t="s">
         <x:v>187</x:v>
-      </x:c>
-      <x:c r="H47" t="s">
-        <x:v>188</x:v>
       </x:c>
       <x:c r="K47" t="s">
         <x:v>52</x:v>
@@ -3362,33 +3371,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U47" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="V47" t="s">
         <x:v>189</x:v>
-      </x:c>
-      <x:c r="V47" t="s">
-        <x:v>190</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="B48" t="s">
         <x:v>193</x:v>
       </x:c>
-      <x:c r="B48" t="s">
+      <x:c r="C48" t="s">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="C48" t="s">
+      <x:c r="D48" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E48" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="D48" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E48" t="s">
+      <x:c r="F48" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="F48" t="s">
+      <x:c r="H48" t="s">
         <x:v>197</x:v>
-      </x:c>
-      <x:c r="H48" t="s">
-        <x:v>198</x:v>
       </x:c>
       <x:c r="K48" t="s">
         <x:v>52</x:v>
@@ -3400,33 +3409,33 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U48" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="V48" t="s">
         <x:v>199</x:v>
-      </x:c>
-      <x:c r="V48" t="s">
-        <x:v>200</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" t="s">
-        <x:v>201</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="B49" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="C49" t="s">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="C49" t="s">
+      <x:c r="D49" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E49" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="D49" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E49" t="s">
+      <x:c r="F49" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="F49" t="s">
+      <x:c r="H49" t="s">
         <x:v>197</x:v>
-      </x:c>
-      <x:c r="H49" t="s">
-        <x:v>198</x:v>
       </x:c>
       <x:c r="K49" t="s">
         <x:v>52</x:v>
@@ -3438,10 +3447,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="U49" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="V49" t="s">
         <x:v>199</x:v>
-      </x:c>
-      <x:c r="V49" t="s">
-        <x:v>200</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3461,7 +3470,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcae7c15e36b4618"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf96762f4b04493e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3485,7 +3494,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>202</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="C1" s="2" t="s">
         <x:v>30</x:v>
@@ -3497,13 +3506,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="F1" s="2" t="s">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="G1" s="2" t="s">
         <x:v>203</x:v>
       </x:c>
-      <x:c r="G1" s="2" t="s">
+      <x:c r="H1" s="3" t="s">
         <x:v>204</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="s">
-        <x:v>205</x:v>
       </x:c>
       <x:c r="I1" t="s">
         <x:v>47</x:v>
@@ -3514,7 +3523,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B2" s="10" t="s">
-        <x:v>206</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="C2" s="4"/>
       <x:c r="D2" s="4"/>
@@ -3523,7 +3532,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G2" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H2" s="11"/>
       <x:c r="I2" t="s">
@@ -3535,7 +3544,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B3" s="10" t="s">
-        <x:v>208</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="C3" s="4"/>
       <x:c r="D3" s="4"/>
@@ -3544,11 +3553,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G3" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H3" s="11"/>
       <x:c r="I3" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -3556,7 +3565,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B4" s="10" t="s">
-        <x:v>209</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="C4" s="4"/>
       <x:c r="D4" s="4"/>
@@ -3565,11 +3574,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H4" s="11"/>
       <x:c r="I4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -3577,7 +3586,7 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B5" s="10" t="s">
-        <x:v>206</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="C5" s="4"/>
       <x:c r="D5" s="4"/>
@@ -3586,7 +3595,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H5" s="11"/>
       <x:c r="I5" t="str">
@@ -3598,7 +3607,7 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B6" s="10" t="s">
-        <x:v>208</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="C6" s="4"/>
       <x:c r="D6" s="4"/>
@@ -3607,11 +3616,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G6" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H6" s="11"/>
       <x:c r="I6" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3619,7 +3628,7 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B7" s="10" t="s">
-        <x:v>209</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="C7" s="4"/>
       <x:c r="D7" s="4"/>
@@ -3628,11 +3637,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H7" s="11"/>
       <x:c r="I7" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -3640,7 +3649,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B8" s="10" t="s">
-        <x:v>206</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="C8" s="4"/>
       <x:c r="D8" s="4"/>
@@ -3649,7 +3658,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G8" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H8" s="11"/>
       <x:c r="I8" t="str">
@@ -3661,7 +3670,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B9" s="10" t="s">
-        <x:v>208</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="C9" s="4"/>
       <x:c r="D9" s="4"/>
@@ -3670,11 +3679,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H9" s="11"/>
       <x:c r="I9" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -3682,7 +3691,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B10" s="10" t="s">
-        <x:v>209</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="C10" s="4"/>
       <x:c r="D10" s="4"/>
@@ -3691,11 +3700,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H10" s="11"/>
       <x:c r="I10" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -3703,7 +3712,7 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B11" s="10" t="s">
-        <x:v>206</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="C11" s="4"/>
       <x:c r="D11" s="4"/>
@@ -3712,7 +3721,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G11" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H11" s="11"/>
       <x:c r="I11" t="str">
@@ -3724,7 +3733,7 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B12" s="10" t="s">
-        <x:v>208</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="C12" s="4"/>
       <x:c r="D12" s="4"/>
@@ -3733,11 +3742,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G12" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H12" s="11"/>
       <x:c r="I12" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -3745,7 +3754,7 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B13" s="10" t="s">
-        <x:v>209</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="C13" s="4"/>
       <x:c r="D13" s="4"/>
@@ -3754,11 +3763,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H13" s="11"/>
       <x:c r="I13" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3772,7 +3781,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re91057a58dc84cc2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93f03117bd6e4c78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3791,87 +3800,87 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="1" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="s">
         <x:v>210</x:v>
       </x:c>
-      <x:c r="B1" s="2" t="s">
+      <x:c r="C1" s="2" t="s">
         <x:v>211</x:v>
       </x:c>
-      <x:c r="C1" s="2" t="s">
-        <x:v>212</x:v>
-      </x:c>
       <x:c r="D1" s="3" t="s">
-        <x:v>205</x:v>
+        <x:v>204</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="B2" s="10" t="s">
         <x:v>213</x:v>
       </x:c>
-      <x:c r="B2" s="10" t="s">
-        <x:v>214</x:v>
-      </x:c>
       <x:c r="C2" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D2" s="4"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="s">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="B3" s="10" t="s">
         <x:v>215</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="s">
-        <x:v>216</x:v>
-      </x:c>
       <x:c r="C3" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D3" s="4"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="10" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="B4" s="10" t="s">
         <x:v>217</x:v>
       </x:c>
-      <x:c r="B4" s="10" t="s">
-        <x:v>218</x:v>
-      </x:c>
       <x:c r="C4" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D4" s="4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="10" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="B5" s="10" t="s">
         <x:v>219</x:v>
       </x:c>
-      <x:c r="B5" s="10" t="s">
-        <x:v>220</x:v>
-      </x:c>
       <x:c r="C5" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D5" s="4"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="10" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="B6" s="10" t="s">
         <x:v>221</x:v>
       </x:c>
-      <x:c r="B6" s="10" t="s">
-        <x:v>222</x:v>
-      </x:c>
       <x:c r="C6" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D6" s="4"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="10" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="B7" s="10" t="s">
         <x:v>223</x:v>
       </x:c>
-      <x:c r="B7" s="10" t="s">
-        <x:v>224</x:v>
-      </x:c>
       <x:c r="C7" s="10" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D7" s="4"/>
     </x:row>
@@ -3883,7 +3892,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b5128ebdcfa4327"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R982107907aec4690"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3905,10 +3914,10 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="s">
         <x:v>225</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="s">
-        <x:v>226</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -3916,115 +3925,115 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="B2" s="10" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="C2" s="11" t="s">
         <x:v>227</x:v>
-      </x:c>
-      <x:c r="C2" s="11" t="s">
-        <x:v>228</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="s">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B3" s="10" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="C3" s="11" t="s">
         <x:v>229</x:v>
-      </x:c>
-      <x:c r="C3" s="11" t="s">
-        <x:v>230</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="10" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="B4" s="10" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="B4" s="10" t="s">
+      <x:c r="C4" s="11" t="s">
         <x:v>232</x:v>
-      </x:c>
-      <x:c r="C4" s="11" t="s">
-        <x:v>233</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="10" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B5" s="10" t="s">
+        <x:v>233</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="s">
         <x:v>234</x:v>
-      </x:c>
-      <x:c r="C5" s="11" t="s">
-        <x:v>235</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="10" t="s">
-        <x:v>106</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B6" s="10" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="s">
         <x:v>236</x:v>
-      </x:c>
-      <x:c r="C6" s="11" t="s">
-        <x:v>237</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="10" t="s">
-        <x:v>114</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="B7" s="10" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="s">
         <x:v>238</x:v>
-      </x:c>
-      <x:c r="C7" s="11" t="s">
-        <x:v>239</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="10" t="s">
-        <x:v>124</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="B8" s="10" t="s">
+        <x:v>239</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="s">
         <x:v>240</x:v>
-      </x:c>
-      <x:c r="C8" s="11" t="s">
-        <x:v>241</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="10" t="s">
-        <x:v>134</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B9" s="10" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="s">
         <x:v>242</x:v>
-      </x:c>
-      <x:c r="C9" s="11" t="s">
-        <x:v>243</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="10" t="s">
+        <x:v>243</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="s">
         <x:v>244</x:v>
       </x:c>
-      <x:c r="B10" s="10" t="s">
+      <x:c r="C10" s="11" t="s">
         <x:v>245</x:v>
-      </x:c>
-      <x:c r="C10" s="11" t="s">
-        <x:v>246</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="s">
-        <x:v>195</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="B11" t="s">
+        <x:v>246</x:v>
+      </x:c>
+      <x:c r="C11" t="s">
         <x:v>247</x:v>
-      </x:c>
-      <x:c r="C11" t="s">
-        <x:v>248</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7508f1a403a4e43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72bd6fef27e9462c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Rename tripod inventory records
</commit_message>
<xml_diff>
--- a/data/templates/NFC_Inventory_Import_Template.xlsx
+++ b/data/templates/NFC_Inventory_Import_Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="Rd1c2b1c46df4453b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="Ra7d675b8b89a4211"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R0d76ad2cdbd541e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="Rf79136a8e59846f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R559ce88da8e348a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R78708799343443e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R1ec2f7575a92469a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R61e768b9a3754cd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="Rb22e291e17f5474d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R63d8785d76c74084"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -278,9 +278,6 @@
     <x:t xml:space="preserve">MNT-003</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Big Tripod</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/victiv-tripod.jpg</x:t>
   </x:si>
   <x:si>
@@ -300,9 +297,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">MNT-008</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Small Tripod</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/lammcou-small-tripod.jpg</x:t>
@@ -2120,8 +2114,8 @@
       <x:c r="A16" s="9" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="B16" s="10" t="s">
-        <x:v>88</x:v>
+      <x:c r="B16" s="10" t="str">
+        <x:v>PEMOTech Tripod</x:v>
       </x:c>
       <x:c r="C16" s="10" t="s">
         <x:v>73</x:v>
@@ -2129,7 +2123,9 @@
       <x:c r="D16" s="10" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E16" s="4"/>
+      <x:c r="E16" s="4" t="str">
+        <x:v>PEMOTech</x:v>
+      </x:c>
       <x:c r="F16" s="4"/>
       <x:c r="G16" s="4"/>
       <x:c r="H16" s="11"/>
@@ -2151,15 +2147,15 @@
       <x:c r="T16" s="11"/>
       <x:c r="U16" s="11"/>
       <x:c r="V16" s="11" t="s">
-        <x:v>89</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="37.5">
       <x:c r="A17" s="9" t="s">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="B17" s="10" t="s">
-        <x:v>88</x:v>
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="str">
+        <x:v>Victiv Tripod</x:v>
       </x:c>
       <x:c r="C17" s="10" t="s">
         <x:v>73</x:v>
@@ -2167,8 +2163,12 @@
       <x:c r="D17" s="10" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E17" s="4"/>
-      <x:c r="F17" s="4"/>
+      <x:c r="E17" s="4" t="str">
+        <x:v>Victiv</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>NT70</x:v>
+      </x:c>
       <x:c r="G17" s="4"/>
       <x:c r="H17" s="11"/>
       <x:c r="I17" s="11"/>
@@ -2189,15 +2189,15 @@
       <x:c r="T17" s="11"/>
       <x:c r="U17" s="11"/>
       <x:c r="V17" s="11" t="s">
-        <x:v>89</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="37.5">
       <x:c r="A18" s="9" t="s">
-        <x:v>91</x:v>
-      </x:c>
-      <x:c r="B18" s="10" t="s">
-        <x:v>88</x:v>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="str">
+        <x:v>K&amp;F Tripod</x:v>
       </x:c>
       <x:c r="C18" s="10" t="s">
         <x:v>73</x:v>
@@ -2205,8 +2205,12 @@
       <x:c r="D18" s="10" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E18" s="4"/>
-      <x:c r="F18" s="4"/>
+      <x:c r="E18" s="4" t="str">
+        <x:v>K&amp;F Concept</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="str">
+        <x:v>K234A0</x:v>
+      </x:c>
       <x:c r="G18" s="4"/>
       <x:c r="H18" s="11"/>
       <x:c r="I18" s="11"/>
@@ -2227,15 +2231,15 @@
       <x:c r="T18" s="11"/>
       <x:c r="U18" s="11"/>
       <x:c r="V18" s="11" t="s">
-        <x:v>89</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="37.5">
       <x:c r="A19" s="9" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="s">
         <x:v>92</x:v>
-      </x:c>
-      <x:c r="B19" s="10" t="s">
-        <x:v>93</x:v>
       </x:c>
       <x:c r="C19" s="10" t="s">
         <x:v>73</x:v>
@@ -2270,10 +2274,10 @@
     </x:row>
     <x:row r="20" ht="37.5">
       <x:c r="A20" s="9" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B20" s="10" t="s">
-        <x:v>93</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C20" s="10" t="s">
         <x:v>73</x:v>
@@ -2308,10 +2312,10 @@
     </x:row>
     <x:row r="21" ht="37.5">
       <x:c r="A21" s="9" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="B21" s="10" t="s">
-        <x:v>96</x:v>
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>Unbranded Three-Stage Tripod</x:v>
       </x:c>
       <x:c r="C21" s="10" t="s">
         <x:v>73</x:v>
@@ -2319,7 +2323,9 @@
       <x:c r="D21" s="10" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E21" s="4"/>
+      <x:c r="E21" s="4" t="str">
+        <x:v>Unbranded</x:v>
+      </x:c>
       <x:c r="F21" s="4"/>
       <x:c r="G21" s="4"/>
       <x:c r="H21" s="11"/>
@@ -2341,15 +2347,15 @@
       <x:c r="T21" s="11"/>
       <x:c r="U21" s="11"/>
       <x:c r="V21" s="11" t="s">
-        <x:v>97</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="37.5">
       <x:c r="A22" s="9" t="s">
-        <x:v>98</x:v>
-      </x:c>
-      <x:c r="B22" s="10" t="s">
         <x:v>96</x:v>
+      </x:c>
+      <x:c r="B22" s="10" t="str">
+        <x:v>Unbranded Three-Stage Tripod</x:v>
       </x:c>
       <x:c r="C22" s="10" t="s">
         <x:v>73</x:v>
@@ -2357,7 +2363,9 @@
       <x:c r="D22" s="10" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E22" s="4"/>
+      <x:c r="E22" s="4" t="str">
+        <x:v>Unbranded</x:v>
+      </x:c>
       <x:c r="F22" s="4"/>
       <x:c r="G22" s="4"/>
       <x:c r="H22" s="11"/>
@@ -2379,15 +2387,15 @@
       <x:c r="T22" s="11"/>
       <x:c r="U22" s="11"/>
       <x:c r="V22" s="11" t="s">
-        <x:v>97</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="37.5">
       <x:c r="A23" s="9" t="s">
-        <x:v>99</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="B23" s="10" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="C23" s="10" t="s">
         <x:v>73</x:v>
@@ -2422,10 +2430,10 @@
     </x:row>
     <x:row r="24" ht="37.5">
       <x:c r="A24" s="9" t="s">
-        <x:v>101</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B24" s="10" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="C24" s="10" t="s">
         <x:v>73</x:v>
@@ -2460,26 +2468,26 @@
     </x:row>
     <x:row r="25" ht="37.5">
       <x:c r="A25" s="9" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="B25" s="10" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="C25" s="10" t="s">
         <x:v>102</x:v>
-      </x:c>
-      <x:c r="B25" s="10" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="C25" s="10" t="s">
-        <x:v>104</x:v>
       </x:c>
       <x:c r="D25" s="10" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E25" s="4" t="s">
-        <x:v>105</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="F25" s="4" t="s">
-        <x:v>106</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="G25" s="4"/>
       <x:c r="H25" s="11" t="s">
-        <x:v>107</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="I25" s="11"/>
       <x:c r="J25" s="11"/>
@@ -2499,31 +2507,31 @@
       <x:c r="T25" s="11"/>
       <x:c r="U25" s="11"/>
       <x:c r="V25" s="11" t="s">
-        <x:v>108</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="37.5">
       <x:c r="A26" s="9" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B26" s="10" t="s">
-        <x:v>103</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C26" s="10" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D26" s="10" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E26" s="4" t="s">
-        <x:v>105</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="F26" s="4" t="s">
-        <x:v>106</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="G26" s="4"/>
       <x:c r="H26" s="11" t="s">
-        <x:v>107</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="I26" s="11"/>
       <x:c r="J26" s="11"/>
@@ -2543,31 +2551,31 @@
       <x:c r="T26" s="11"/>
       <x:c r="U26" s="11"/>
       <x:c r="V26" s="11" t="s">
-        <x:v>108</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="37.5">
       <x:c r="A27" s="9" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="B27" s="10" t="s">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="C27" s="10" t="s">
         <x:v>110</x:v>
-      </x:c>
-      <x:c r="B27" s="10" t="s">
-        <x:v>111</x:v>
-      </x:c>
-      <x:c r="C27" s="10" t="s">
-        <x:v>112</x:v>
       </x:c>
       <x:c r="D27" s="10" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E27" s="4" t="s">
-        <x:v>113</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="F27" s="4" t="s">
-        <x:v>114</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="G27" s="4"/>
       <x:c r="H27" s="11" t="s">
-        <x:v>115</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="I27" s="11"/>
       <x:c r="J27" s="11"/>
@@ -2587,18 +2595,18 @@
       <x:c r="T27" s="11"/>
       <x:c r="U27" s="11"/>
       <x:c r="V27" s="11" t="s">
-        <x:v>116</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="37.5">
       <x:c r="A28" s="9" t="s">
-        <x:v>117</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="B28" s="10" t="s">
-        <x:v>118</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="C28" s="10" t="s">
-        <x:v>112</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="D28" s="10" t="s">
         <x:v>50</x:v>
@@ -2625,18 +2633,18 @@
       <x:c r="T28" s="11"/>
       <x:c r="U28" s="11"/>
       <x:c r="V28" s="11" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="37.5">
       <x:c r="A29" s="9" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="B29" s="10" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="C29" s="10" t="s">
         <x:v>120</x:v>
-      </x:c>
-      <x:c r="B29" s="10" t="s">
-        <x:v>121</x:v>
-      </x:c>
-      <x:c r="C29" s="10" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="D29" s="10" t="s">
         <x:v>50</x:v>
@@ -2668,13 +2676,13 @@
     </x:row>
     <x:row r="30" ht="37.5">
       <x:c r="A30" s="9" t="s">
-        <x:v>123</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B30" s="10" t="s">
-        <x:v>121</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C30" s="10" t="s">
-        <x:v>122</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="D30" s="10" t="s">
         <x:v>50</x:v>
@@ -2706,13 +2714,13 @@
     </x:row>
     <x:row r="31" ht="37.5">
       <x:c r="A31" s="9" t="s">
-        <x:v>124</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B31" s="10" t="s">
-        <x:v>125</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="C31" s="10" t="s">
-        <x:v>122</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="D31" s="10" t="s">
         <x:v>50</x:v>
@@ -2739,18 +2747,18 @@
       <x:c r="T31" s="11"/>
       <x:c r="U31" s="11"/>
       <x:c r="V31" s="11" t="s">
-        <x:v>126</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="37.5">
       <x:c r="A32" s="9" t="s">
-        <x:v>127</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B32" s="10" t="s">
-        <x:v>128</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C32" s="10" t="s">
-        <x:v>122</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="D32" s="10" t="s">
         <x:v>50</x:v>
@@ -2777,31 +2785,31 @@
       <x:c r="T32" s="11"/>
       <x:c r="U32" s="11"/>
       <x:c r="V32" s="11" t="s">
-        <x:v>129</x:v>
+        <x:v>127</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="87.5">
       <x:c r="A33" s="9" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="B33" s="10" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="C33" s="10" t="s">
         <x:v>130</x:v>
-      </x:c>
-      <x:c r="B33" s="10" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="C33" s="10" t="s">
-        <x:v>132</x:v>
       </x:c>
       <x:c r="D33" s="10" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E33" s="4" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="F33" s="4" t="s">
-        <x:v>134</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="G33" s="4"/>
       <x:c r="H33" s="11" t="s">
-        <x:v>135</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="I33" s="11"/>
       <x:c r="J33" s="11"/>
@@ -2822,34 +2830,34 @@
       <x:c r="S33" s="11"/>
       <x:c r="T33" s="11"/>
       <x:c r="U33" s="11" t="s">
-        <x:v>136</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="V33" s="11" t="s">
-        <x:v>137</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="87.5">
       <x:c r="A34" s="9" t="s">
-        <x:v>138</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="B34" s="10" t="s">
-        <x:v>131</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="C34" s="10" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D34" s="10" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E34" s="4" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="F34" s="4" t="s">
-        <x:v>134</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="G34" s="4"/>
       <x:c r="H34" s="11" t="s">
-        <x:v>135</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="I34" s="11"/>
       <x:c r="J34" s="11"/>
@@ -2870,18 +2878,18 @@
       <x:c r="S34" s="11"/>
       <x:c r="T34" s="11"/>
       <x:c r="U34" s="11" t="s">
-        <x:v>136</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="V34" s="11" t="s">
-        <x:v>137</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B35" t="s">
-        <x:v>140</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C35" t="str">
         <x:v>Cameras</x:v>
@@ -2890,13 +2898,13 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="E35" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="F35" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="H35" t="s">
         <x:v>141</x:v>
-      </x:c>
-      <x:c r="F35" t="s">
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="H35" t="s">
-        <x:v>143</x:v>
       </x:c>
       <x:c r="K35" t="s">
         <x:v>51</x:v>
@@ -2908,18 +2916,18 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U35" t="s">
-        <x:v>144</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="V35" t="s">
-        <x:v>145</x:v>
+        <x:v>143</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="s">
-        <x:v>146</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="B36" t="s">
-        <x:v>147</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="C36" t="str">
         <x:v>Cameras</x:v>
@@ -2928,13 +2936,13 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="E36" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="F36" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="H36" t="s">
         <x:v>148</x:v>
-      </x:c>
-      <x:c r="F36" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="H36" t="s">
-        <x:v>150</x:v>
       </x:c>
       <x:c r="K36" t="s">
         <x:v>51</x:v>
@@ -2946,18 +2954,18 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U36" t="s">
-        <x:v>151</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="V36" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="s">
-        <x:v>153</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B37" t="s">
-        <x:v>154</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="C37" t="s">
         <x:v>68</x:v>
@@ -2966,13 +2974,13 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="E37" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="F37" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="H37" t="s">
         <x:v>155</x:v>
-      </x:c>
-      <x:c r="F37" t="s">
-        <x:v>156</x:v>
-      </x:c>
-      <x:c r="H37" t="s">
-        <x:v>157</x:v>
       </x:c>
       <x:c r="K37" t="s">
         <x:v>51</x:v>
@@ -2984,18 +2992,18 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U37" t="s">
-        <x:v>158</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="V37" t="s">
-        <x:v>159</x:v>
+        <x:v>157</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="s">
-        <x:v>160</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B38" t="s">
-        <x:v>154</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="C38" t="s">
         <x:v>68</x:v>
@@ -3004,13 +3012,13 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="E38" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="F38" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="H38" t="s">
         <x:v>155</x:v>
-      </x:c>
-      <x:c r="F38" t="s">
-        <x:v>156</x:v>
-      </x:c>
-      <x:c r="H38" t="s">
-        <x:v>157</x:v>
       </x:c>
       <x:c r="K38" t="s">
         <x:v>51</x:v>
@@ -3022,18 +3030,18 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U38" t="s">
-        <x:v>158</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="V38" t="s">
-        <x:v>159</x:v>
+        <x:v>157</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" t="s">
-        <x:v>161</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B39" t="s">
-        <x:v>162</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C39" t="s">
         <x:v>68</x:v>
@@ -3042,13 +3050,13 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="E39" t="s">
-        <x:v>155</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="F39" t="s">
-        <x:v>163</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="H39" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="K39" t="s">
         <x:v>51</x:v>
@@ -3060,18 +3068,18 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U39" t="s">
-        <x:v>165</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="V39" t="s">
-        <x:v>166</x:v>
+        <x:v>164</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" t="s">
-        <x:v>167</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B40" t="s">
-        <x:v>168</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="C40" t="s">
         <x:v>73</x:v>
@@ -3080,10 +3088,10 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="F40" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="H40" t="s">
-        <x:v>170</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="K40" t="s">
         <x:v>51</x:v>
@@ -3095,7 +3103,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U40" t="s">
-        <x:v>171</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="V40" t="s">
         <x:v>69</x:v>
@@ -3103,25 +3111,25 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" t="s">
-        <x:v>172</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B41" t="s">
-        <x:v>131</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="C41" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D41" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E41" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="F41" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="H41" t="s">
         <x:v>133</x:v>
-      </x:c>
-      <x:c r="F41" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="H41" t="s">
-        <x:v>135</x:v>
       </x:c>
       <x:c r="K41" t="s">
         <x:v>51</x:v>
@@ -3133,33 +3141,33 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U41" t="s">
-        <x:v>136</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="V41" t="s">
-        <x:v>137</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" t="s">
-        <x:v>173</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B42" t="s">
-        <x:v>174</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="C42" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D42" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E42" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="F42" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="H42" t="s">
         <x:v>175</x:v>
-      </x:c>
-      <x:c r="F42" t="s">
-        <x:v>176</x:v>
-      </x:c>
-      <x:c r="H42" t="s">
-        <x:v>177</x:v>
       </x:c>
       <x:c r="K42" t="s">
         <x:v>51</x:v>
@@ -3171,33 +3179,33 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U42" t="s">
-        <x:v>178</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="V42" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" t="s">
-        <x:v>180</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B43" t="s">
-        <x:v>174</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="C43" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D43" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E43" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="F43" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="H43" t="s">
         <x:v>175</x:v>
-      </x:c>
-      <x:c r="F43" t="s">
-        <x:v>176</x:v>
-      </x:c>
-      <x:c r="H43" t="s">
-        <x:v>177</x:v>
       </x:c>
       <x:c r="K43" t="s">
         <x:v>51</x:v>
@@ -3209,33 +3217,33 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U43" t="s">
-        <x:v>178</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="V43" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" t="s">
-        <x:v>181</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B44" t="s">
-        <x:v>174</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="C44" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D44" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E44" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="F44" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="H44" t="s">
         <x:v>175</x:v>
-      </x:c>
-      <x:c r="F44" t="s">
-        <x:v>176</x:v>
-      </x:c>
-      <x:c r="H44" t="s">
-        <x:v>177</x:v>
       </x:c>
       <x:c r="K44" t="s">
         <x:v>51</x:v>
@@ -3247,33 +3255,33 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U44" t="s">
-        <x:v>178</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="V44" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" t="s">
-        <x:v>182</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="B45" t="s">
-        <x:v>183</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="C45" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D45" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E45" t="s">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="F45" t="s">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="H45" t="s">
         <x:v>184</x:v>
-      </x:c>
-      <x:c r="F45" t="s">
-        <x:v>185</x:v>
-      </x:c>
-      <x:c r="H45" t="s">
-        <x:v>186</x:v>
       </x:c>
       <x:c r="K45" t="s">
         <x:v>51</x:v>
@@ -3285,33 +3293,33 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U45" t="s">
-        <x:v>187</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="V45" t="s">
-        <x:v>188</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" t="s">
-        <x:v>189</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B46" t="s">
-        <x:v>183</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="C46" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D46" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E46" t="s">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="F46" t="s">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="H46" t="s">
         <x:v>184</x:v>
-      </x:c>
-      <x:c r="F46" t="s">
-        <x:v>185</x:v>
-      </x:c>
-      <x:c r="H46" t="s">
-        <x:v>186</x:v>
       </x:c>
       <x:c r="K46" t="s">
         <x:v>51</x:v>
@@ -3323,33 +3331,33 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U46" t="s">
-        <x:v>187</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="V46" t="s">
-        <x:v>188</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" t="s">
-        <x:v>190</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="B47" t="s">
-        <x:v>183</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="C47" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D47" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E47" t="s">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="F47" t="s">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="H47" t="s">
         <x:v>184</x:v>
-      </x:c>
-      <x:c r="F47" t="s">
-        <x:v>185</x:v>
-      </x:c>
-      <x:c r="H47" t="s">
-        <x:v>186</x:v>
       </x:c>
       <x:c r="K47" t="s">
         <x:v>51</x:v>
@@ -3361,33 +3369,33 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U47" t="s">
-        <x:v>187</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="V47" t="s">
-        <x:v>188</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" t="s">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="B48" t="s">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="C48" t="s">
         <x:v>191</x:v>
-      </x:c>
-      <x:c r="B48" t="s">
-        <x:v>192</x:v>
-      </x:c>
-      <x:c r="C48" t="s">
-        <x:v>193</x:v>
       </x:c>
       <x:c r="D48" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E48" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="F48" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="H48" t="s">
         <x:v>194</x:v>
-      </x:c>
-      <x:c r="F48" t="s">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="H48" t="s">
-        <x:v>196</x:v>
       </x:c>
       <x:c r="K48" t="s">
         <x:v>51</x:v>
@@ -3399,33 +3407,33 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U48" t="s">
-        <x:v>197</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="V48" t="s">
-        <x:v>198</x:v>
+        <x:v>196</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" t="s">
-        <x:v>199</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="B49" t="s">
-        <x:v>192</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="C49" t="s">
-        <x:v>193</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="D49" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E49" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="F49" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="H49" t="s">
         <x:v>194</x:v>
-      </x:c>
-      <x:c r="F49" t="s">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="H49" t="s">
-        <x:v>196</x:v>
       </x:c>
       <x:c r="K49" t="s">
         <x:v>51</x:v>
@@ -3437,10 +3445,10 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="U49" t="s">
-        <x:v>197</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="V49" t="s">
-        <x:v>198</x:v>
+        <x:v>196</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -4769,7 +4777,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dfef7f8f8154cc6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recc76ca8e5ee4aed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4793,7 +4801,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>200</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C1" s="2" t="s">
         <x:v>29</x:v>
@@ -4805,13 +4813,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="F1" s="2" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="G1" s="2" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="H1" s="3" t="s">
         <x:v>201</x:v>
-      </x:c>
-      <x:c r="G1" s="2" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="s">
-        <x:v>203</x:v>
       </x:c>
       <x:c r="I1" t="s">
         <x:v>46</x:v>
@@ -5548,7 +5556,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb82a3c10c7f4486e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35e8a9f14c884c46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5567,87 +5575,87 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="1" t="s">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="C1" s="2" t="s">
         <x:v>204</x:v>
       </x:c>
-      <x:c r="B1" s="2" t="s">
-        <x:v>205</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="s">
-        <x:v>206</x:v>
-      </x:c>
       <x:c r="D1" s="3" t="s">
-        <x:v>203</x:v>
+        <x:v>201</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="10" t="s">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="B2" s="10" t="s">
+        <x:v>206</x:v>
+      </x:c>
+      <x:c r="C2" s="10" t="s">
         <x:v>207</x:v>
-      </x:c>
-      <x:c r="B2" s="10" t="s">
-        <x:v>208</x:v>
-      </x:c>
-      <x:c r="C2" s="10" t="s">
-        <x:v>209</x:v>
       </x:c>
       <x:c r="D2" s="4"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="s">
-        <x:v>210</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="B3" s="10" t="s">
-        <x:v>211</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="C3" s="10" t="s">
-        <x:v>209</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="D3" s="4"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="10" t="s">
-        <x:v>212</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="B4" s="10" t="s">
-        <x:v>213</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C4" s="10" t="s">
-        <x:v>209</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="D4" s="4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="10" t="s">
-        <x:v>214</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="B5" s="10" t="s">
-        <x:v>215</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="C5" s="10" t="s">
-        <x:v>209</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="D5" s="4"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="10" t="s">
-        <x:v>216</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="B6" s="10" t="s">
-        <x:v>217</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="C6" s="10" t="s">
-        <x:v>209</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="D6" s="4"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="10" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B7" s="10" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="C7" s="10" t="s">
-        <x:v>209</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="D7" s="4"/>
     </x:row>
@@ -5659,7 +5667,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a5445168ddc404b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf529312bef6140b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5681,10 +5689,10 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>220</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C1" s="3" t="s">
-        <x:v>221</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -5692,10 +5700,10 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B2" s="10" t="s">
-        <x:v>222</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="C2" s="11" t="s">
-        <x:v>223</x:v>
+        <x:v>221</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -5703,21 +5711,21 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B3" s="10" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="C3" s="11" t="s">
-        <x:v>225</x:v>
+        <x:v>223</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="10" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="B4" s="10" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="s">
         <x:v>226</x:v>
-      </x:c>
-      <x:c r="B4" s="10" t="s">
-        <x:v>227</x:v>
-      </x:c>
-      <x:c r="C4" s="11" t="s">
-        <x:v>228</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -5725,76 +5733,76 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B5" s="10" t="s">
-        <x:v>229</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="C5" s="11" t="s">
-        <x:v>230</x:v>
+        <x:v>228</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="10" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B6" s="10" t="s">
-        <x:v>231</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="C6" s="11" t="s">
-        <x:v>232</x:v>
+        <x:v>230</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="10" t="s">
-        <x:v>112</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B7" s="10" t="s">
-        <x:v>233</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="C7" s="11" t="s">
-        <x:v>234</x:v>
+        <x:v>232</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="10" t="s">
-        <x:v>122</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B8" s="10" t="s">
-        <x:v>235</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="C8" s="11" t="s">
-        <x:v>236</x:v>
+        <x:v>234</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="10" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="B9" s="10" t="s">
-        <x:v>237</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C9" s="11" t="s">
-        <x:v>238</x:v>
+        <x:v>236</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="10" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="s">
         <x:v>239</x:v>
-      </x:c>
-      <x:c r="B10" s="10" t="s">
-        <x:v>240</x:v>
-      </x:c>
-      <x:c r="C10" s="11" t="s">
-        <x:v>241</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="s">
-        <x:v>193</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="B11" t="s">
-        <x:v>242</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="C11" t="s">
-        <x:v>243</x:v>
+        <x:v>241</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -5833,7 +5841,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1965319964e7468b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde40156dd5e1433b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct ROB-006 to wireless model
</commit_message>
<xml_diff>
--- a/data/templates/NFC_Inventory_Import_Template.xlsx
+++ b/data/templates/NFC_Inventory_Import_Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R78708799343443e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R1ec2f7575a92469a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R61e768b9a3754cd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="Rb22e291e17f5474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R63d8785d76c74084"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R2ab823917c754294"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R2f811497a6d14128"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="Re52e61fe6f244595"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="R861d94f5bf4b42b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="Rbdfb56e206fd40cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1736,8 +1736,8 @@
       <x:c r="A7" s="9" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="B7" s="10" t="s">
-        <x:v>62</x:v>
+      <x:c r="B7" s="10" t="str">
+        <x:v>Reachy Mini Wireless</x:v>
       </x:c>
       <x:c r="C7" s="10" t="s">
         <x:v>49</x:v>
@@ -1748,11 +1748,13 @@
       <x:c r="E7" s="4" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="F7" s="4" t="s">
-        <x:v>62</x:v>
+      <x:c r="F7" s="4" t="str">
+        <x:v>Reachy Mini Wireless</x:v>
       </x:c>
       <x:c r="G7" s="4"/>
-      <x:c r="H7" s="11"/>
+      <x:c r="H7" s="11" t="str">
+        <x:v>Wireless Reachy Mini robot bundle</x:v>
+      </x:c>
       <x:c r="I7" s="11"/>
       <x:c r="J7" s="11"/>
       <x:c r="K7" s="12" t="s">
@@ -1770,8 +1772,8 @@
       <x:c r="S7" s="11"/>
       <x:c r="T7" s="11"/>
       <x:c r="U7" s="11"/>
-      <x:c r="V7" s="11" t="s">
-        <x:v>64</x:v>
+      <x:c r="V7" s="11" t="str">
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-wireless.png</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="37.5">
@@ -4777,7 +4779,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recc76ca8e5ee4aed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3b45ed2e1424ab3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5037,7 +5039,7 @@
         <x:v>Pollen Robotics</x:v>
       </x:c>
       <x:c r="D11" s="4" t="str">
-        <x:v>Reachy Mini Lite</x:v>
+        <x:v>Reachy Mini Wireless</x:v>
       </x:c>
       <x:c r="E11" s="4"/>
       <x:c r="F11" s="10" t="n">
@@ -5048,7 +5050,7 @@
       </x:c>
       <x:c r="H11" s="11"/>
       <x:c r="I11" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-lite.png</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-wireless.png</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -5556,7 +5558,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35e8a9f14c884c46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcf6dd3a50754133"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5667,7 +5669,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf529312bef6140b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb078d135983444b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5841,7 +5843,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde40156dd5e1433b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a356ff9ed5c4848"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add two DJI Mic 3 transmitters
</commit_message>
<xml_diff>
--- a/data/templates/NFC_Inventory_Import_Template.xlsx
+++ b/data/templates/NFC_Inventory_Import_Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R825b30ce035344b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R50c028b5084544b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="Rd4c794bb905244c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="R8b73a9e01e534673"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R9e247bb6e2274f25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R1be9b515e85a47a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R5921a656f590438b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="Re5dfcdaa88734f42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="Race9fedfdab5486f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R30e0a418c9a04711"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -508,8 +508,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EquipmentTable" displayName="EquipmentTable" ref="A1:V79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:V79"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EquipmentTable" displayName="EquipmentTable" ref="A1:V81" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:V81"/>
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="asset_code"/>
     <x:tableColumn id="2" name="equipment_name"/>
@@ -824,7 +824,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>77 unique equipment units are included. One asset code is used for each physical unit or complete bundle.</x:v>
+        <x:v>79 unique equipment units are included. One asset code is used for each physical unit or complete bundle.</x:v>
       </x:c>
       <x:c r="C4" s="4"/>
       <x:c r="D4" s="4"/>
@@ -4434,20 +4434,38 @@
       </x:c>
     </x:row>
     <x:row r="79">
-      <x:c r="A79"/>
-      <x:c r="B79"/>
-      <x:c r="C79"/>
-      <x:c r="D79"/>
-      <x:c r="E79"/>
-      <x:c r="F79"/>
+      <x:c r="A79" t="str">
+        <x:v>AUD-003</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>DJI Mic 3 Transmitter</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>Audio equipment</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>Individual</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>DJI</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>DMT03</x:v>
+      </x:c>
       <x:c r="G79"/>
-      <x:c r="H79"/>
+      <x:c r="H79" t="str">
+        <x:v>Wireless microphone transmitter; 32-bit float/24-bit internal recording, 32 GB storage, Bluetooth 5.4 and up to 8-hour operation</x:v>
+      </x:c>
       <x:c r="I79"/>
       <x:c r="J79"/>
-      <x:c r="K79"/>
+      <x:c r="K79" t="str">
+        <x:v>Active</x:v>
+      </x:c>
       <x:c r="L79"/>
       <x:c r="M79"/>
-      <x:c r="N79"/>
+      <x:c r="N79" t="str">
+        <x:v>GBP</x:v>
+      </x:c>
       <x:c r="O79"/>
       <x:c r="P79"/>
       <x:c r="Q79"/>
@@ -4455,7 +4473,77 @@
       <x:c r="S79"/>
       <x:c r="T79"/>
       <x:c r="U79"/>
-      <x:c r="V79"/>
+      <x:c r="V79" t="str">
+        <x:v>https://se-cdn.djiits.com/tpc/uploads/spu/cover/5ac37a6cf8ca7e9e01c18dd9fc096fe8%40small.png?format=webp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>AUD-004</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>DJI Mic 3 Transmitter</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>Audio equipment</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>Individual</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>DJI</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>DMT03</x:v>
+      </x:c>
+      <x:c r="G80"/>
+      <x:c r="H80" t="str">
+        <x:v>Wireless microphone transmitter; 32-bit float/24-bit internal recording, 32 GB storage, Bluetooth 5.4 and up to 8-hour operation</x:v>
+      </x:c>
+      <x:c r="I80"/>
+      <x:c r="J80"/>
+      <x:c r="K80" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="L80"/>
+      <x:c r="M80"/>
+      <x:c r="N80" t="str">
+        <x:v>GBP</x:v>
+      </x:c>
+      <x:c r="O80"/>
+      <x:c r="P80"/>
+      <x:c r="Q80"/>
+      <x:c r="R80"/>
+      <x:c r="S80"/>
+      <x:c r="T80"/>
+      <x:c r="U80"/>
+      <x:c r="V80" t="str">
+        <x:v>https://se-cdn.djiits.com/tpc/uploads/spu/cover/5ac37a6cf8ca7e9e01c18dd9fc096fe8%40small.png?format=webp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81"/>
+      <x:c r="B81"/>
+      <x:c r="C81"/>
+      <x:c r="D81"/>
+      <x:c r="E81"/>
+      <x:c r="F81"/>
+      <x:c r="G81"/>
+      <x:c r="H81"/>
+      <x:c r="I81"/>
+      <x:c r="J81"/>
+      <x:c r="K81"/>
+      <x:c r="L81"/>
+      <x:c r="M81"/>
+      <x:c r="N81"/>
+      <x:c r="O81"/>
+      <x:c r="P81"/>
+      <x:c r="Q81"/>
+      <x:c r="R81"/>
+      <x:c r="S81"/>
+      <x:c r="T81"/>
+      <x:c r="U81"/>
+      <x:c r="V81"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="5">
@@ -4477,7 +4565,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b1006f76e924a01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3047bf5b53d4886"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5256,7 +5344,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4281346b77d947fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00d18770f38f4c0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5367,7 +5455,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcb593d5602a4751"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75e21adb1ff64988"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5541,7 +5629,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf5e125fad024d6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb49f1abc9e0848f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Naimeh as active member
</commit_message>
<xml_diff>
--- a/data/templates/NFC_Inventory_Import_Template.xlsx
+++ b/data/templates/NFC_Inventory_Import_Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R1be9b515e85a47a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R5921a656f590438b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="Re5dfcdaa88734f42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="Race9fedfdab5486f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R30e0a418c9a04711"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="Rdf3cfd2e609f40a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="Rb1372ea0635b4219"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R5d867cb2a2524b48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="Rabf45558dd3942f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R1b0c3d6972834e81"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -557,8 +557,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="MembersTable" displayName="MembersTable" ref="A1:D7" totalsRowShown="0">
-  <x:autoFilter ref="A1:D7"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="MembersTable" displayName="MembersTable" ref="A1:D8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:D8"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="username"/>
     <x:tableColumn id="2" name="display_name"/>
@@ -4565,7 +4565,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3047bf5b53d4886"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11450d08c6664261"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5344,7 +5344,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00d18770f38f4c0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fa08336730b48b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5447,6 +5447,18 @@
       </x:c>
       <x:c r="D7" s="4"/>
     </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>naimeh.fakhr-vaezi25</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Naimeh</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D8"/>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C2:C7">
@@ -5455,7 +5467,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75e21adb1ff64988"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31aed7fdeb2e4633"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5629,7 +5641,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb49f1abc9e0848f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f89ac8cdb7c4ffb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add DJI Mic 3 set
</commit_message>
<xml_diff>
--- a/data/templates/NFC_Inventory_Import_Template.xlsx
+++ b/data/templates/NFC_Inventory_Import_Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="Rdf3cfd2e609f40a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="Rb1372ea0635b4219"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R5d867cb2a2524b48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="Rabf45558dd3942f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R1b0c3d6972834e81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R163bc0692e304949"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="Rb602d8c0fe4f46f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="Rf03e4402a5f246b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="Re32920b2b3184301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="Rffaf204d6896427b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4522,20 +4522,38 @@
       </x:c>
     </x:row>
     <x:row r="81">
-      <x:c r="A81"/>
-      <x:c r="B81"/>
-      <x:c r="C81"/>
-      <x:c r="D81"/>
-      <x:c r="E81"/>
-      <x:c r="F81"/>
+      <x:c r="A81" t="str">
+        <x:v>AUD-005</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>DJI Mic 3 Set</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>Audio equipment</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>Individual</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>DJI</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>DJI Mic 3 (2 TX + 1 RX)</x:v>
+      </x:c>
       <x:c r="G81"/>
-      <x:c r="H81"/>
+      <x:c r="H81" t="str">
+        <x:v>Wireless microphone set with one receiver, two transmitters and charging case; 32-bit float/24-bit recording, 400 m maximum transmission range and up to 28-hour operation with case</x:v>
+      </x:c>
       <x:c r="I81"/>
       <x:c r="J81"/>
-      <x:c r="K81"/>
+      <x:c r="K81" t="str">
+        <x:v>Active</x:v>
+      </x:c>
       <x:c r="L81"/>
       <x:c r="M81"/>
-      <x:c r="N81"/>
+      <x:c r="N81" t="str">
+        <x:v>GBP</x:v>
+      </x:c>
       <x:c r="O81"/>
       <x:c r="P81"/>
       <x:c r="Q81"/>
@@ -4543,7 +4561,9 @@
       <x:c r="S81"/>
       <x:c r="T81"/>
       <x:c r="U81"/>
-      <x:c r="V81"/>
+      <x:c r="V81" t="str">
+        <x:v>https://se-cdn.djiits.com/tpc/uploads/spu/cover/473691cc5e140d0341a30b31b479c627%40small.png?format=webp</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="5">
@@ -4565,7 +4585,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11450d08c6664261"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d4115b8e82f40f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5344,7 +5364,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fa08336730b48b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39a9becd9f514c35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5467,7 +5487,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31aed7fdeb2e4633"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35ccca0549894800"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5641,7 +5661,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f89ac8cdb7c4ffb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88b6b225f2844c98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct ROB-003 and ROB-005 inventory records
</commit_message>
<xml_diff>
--- a/data/templates/NFC_Inventory_Import_Template.xlsx
+++ b/data/templates/NFC_Inventory_Import_Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R163bc0692e304949"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="Rb602d8c0fe4f46f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="Rf03e4402a5f246b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="Re32920b2b3184301"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="Rffaf204d6896427b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="Rb357be9528194c38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R8d9308c0e0074fc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle contents" sheetId="3" r:id="R4ad25641f56a4c2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="4" r:id="R6bcd363f104841ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="5" r:id="R432f5b42b1d9497a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1172,31 +1172,25 @@
         <x:v>ROB-003</x:v>
       </x:c>
       <x:c r="B4" s="10" t="str">
-        <x:v>Reachy Mini Wireless</x:v>
+        <x:v>NAO Robot</x:v>
       </x:c>
       <x:c r="C4" s="10" t="str">
         <x:v>Robots</x:v>
       </x:c>
       <x:c r="D4" s="10" t="str">
-        <x:v>Bundle</x:v>
-      </x:c>
-      <x:c r="E4" s="4" t="str">
-        <x:v>Pollen Robotics</x:v>
-      </x:c>
-      <x:c r="F4" s="4" t="str">
-        <x:v>Reachy Mini Wireless</x:v>
-      </x:c>
+        <x:v>Individual</x:v>
+      </x:c>
+      <x:c r="E4" s="4"/>
+      <x:c r="F4" s="4"/>
       <x:c r="G4" s="4"/>
       <x:c r="H4" s="11"/>
       <x:c r="I4" s="11"/>
       <x:c r="J4" s="11"/>
       <x:c r="K4" s="12" t="str">
-        <x:v>Active</x:v>
+        <x:v>Retired</x:v>
       </x:c>
       <x:c r="L4" s="13"/>
-      <x:c r="M4" s="14" t="n">
-        <x:v>439.93</x:v>
-      </x:c>
+      <x:c r="M4" s="14"/>
       <x:c r="N4" s="11" t="str">
         <x:v>GBP</x:v>
       </x:c>
@@ -1206,11 +1200,9 @@
       <x:c r="R4" s="11"/>
       <x:c r="S4" s="11"/>
       <x:c r="T4" s="11"/>
-      <x:c r="U4" s="11" t="str">
-        <x:v>SQ550205 / REACHY-MIN-WLS</x:v>
-      </x:c>
+      <x:c r="U4" s="11"/>
       <x:c r="V4" s="11" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-wireless.png</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="37.5">
@@ -1279,16 +1271,16 @@
         <x:v>Reachy Mini Wireless</x:v>
       </x:c>
       <x:c r="G6" s="4"/>
-      <x:c r="H6" s="11" t="str">
-        <x:v>Wireless Reachy Mini robot bundle</x:v>
-      </x:c>
+      <x:c r="H6" s="11"/>
       <x:c r="I6" s="11"/>
       <x:c r="J6" s="11"/>
       <x:c r="K6" s="12" t="str">
         <x:v>Active</x:v>
       </x:c>
       <x:c r="L6" s="13"/>
-      <x:c r="M6" s="14"/>
+      <x:c r="M6" s="14" t="n">
+        <x:v>439.93</x:v>
+      </x:c>
       <x:c r="N6" s="11" t="str">
         <x:v>GBP</x:v>
       </x:c>
@@ -1298,7 +1290,9 @@
       <x:c r="R6" s="11"/>
       <x:c r="S6" s="11"/>
       <x:c r="T6" s="11"/>
-      <x:c r="U6" s="11"/>
+      <x:c r="U6" s="11" t="str">
+        <x:v>SQ550205 / REACHY-MIN-WLS</x:v>
+      </x:c>
       <x:c r="V6" s="11" t="str">
         <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-wireless.png</x:v>
       </x:c>
@@ -4585,7 +4579,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d4115b8e82f40f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d95a47ebcc64f96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4635,7 +4629,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="10" t="str">
-        <x:v>ROB-003</x:v>
+        <x:v>ROB-004</x:v>
       </x:c>
       <x:c r="B2" s="10" t="str">
         <x:v>Robot</x:v>
@@ -4644,7 +4638,7 @@
         <x:v>Pollen Robotics</x:v>
       </x:c>
       <x:c r="D2" s="4" t="str">
-        <x:v>Reachy Mini Wireless</x:v>
+        <x:v>Reachy Mini Lite</x:v>
       </x:c>
       <x:c r="E2" s="4"/>
       <x:c r="F2" s="10" t="n">
@@ -4655,12 +4649,12 @@
       </x:c>
       <x:c r="H2" s="11"/>
       <x:c r="I2" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-wireless.png</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-lite.png</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
-        <x:v>ROB-003</x:v>
+        <x:v>ROB-004</x:v>
       </x:c>
       <x:c r="B3" s="10" t="str">
         <x:v>Charger</x:v>
@@ -4681,7 +4675,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="10" t="str">
-        <x:v>ROB-003</x:v>
+        <x:v>ROB-004</x:v>
       </x:c>
       <x:c r="B4" s="10" t="str">
         <x:v>USB Cable</x:v>
@@ -4702,7 +4696,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="10" t="str">
-        <x:v>ROB-004</x:v>
+        <x:v>ROB-005</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
         <x:v>Robot</x:v>
@@ -4711,7 +4705,7 @@
         <x:v>Pollen Robotics</x:v>
       </x:c>
       <x:c r="D5" s="4" t="str">
-        <x:v>Reachy Mini Lite</x:v>
+        <x:v>Reachy Mini Wireless</x:v>
       </x:c>
       <x:c r="E5" s="4"/>
       <x:c r="F5" s="10" t="n">
@@ -4722,12 +4716,12 @@
       </x:c>
       <x:c r="H5" s="11"/>
       <x:c r="I5" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-lite.png</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-wireless.png</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="10" t="str">
-        <x:v>ROB-004</x:v>
+        <x:v>ROB-005</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
         <x:v>Charger</x:v>
@@ -4748,7 +4742,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="10" t="str">
-        <x:v>ROB-004</x:v>
+        <x:v>ROB-005</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
         <x:v>USB Cable</x:v>
@@ -4769,7 +4763,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="10" t="str">
-        <x:v>ROB-005</x:v>
+        <x:v>ROB-006</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
         <x:v>Robot</x:v>
@@ -4794,7 +4788,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="10" t="str">
-        <x:v>ROB-005</x:v>
+        <x:v>ROB-006</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
         <x:v>Charger</x:v>
@@ -4815,7 +4809,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="10" t="str">
-        <x:v>ROB-005</x:v>
+        <x:v>ROB-006</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
         <x:v>USB Cable</x:v>
@@ -4836,7 +4830,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="10" t="str">
-        <x:v>ROB-006</x:v>
+        <x:v>ROB-007</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
         <x:v>Robot</x:v>
@@ -4861,7 +4855,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="10" t="str">
-        <x:v>ROB-006</x:v>
+        <x:v>ROB-007</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
         <x:v>Charger</x:v>
@@ -4882,7 +4876,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="10" t="str">
-        <x:v>ROB-006</x:v>
+        <x:v>ROB-007</x:v>
       </x:c>
       <x:c r="B13" s="10" t="str">
         <x:v>USB Cable</x:v>
@@ -4903,16 +4897,16 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>ROB-007</x:v>
+        <x:v>PER-001</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>Robot</x:v>
+        <x:v>Keyboard</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>Pollen Robotics</x:v>
+        <x:v>Logitech</x:v>
       </x:c>
       <x:c r="D14" t="str">
-        <x:v>Reachy Mini Wireless</x:v>
+        <x:v>MK270</x:v>
       </x:c>
       <x:c r="E14"/>
       <x:c r="F14" t="n">
@@ -4923,18 +4917,22 @@
       </x:c>
       <x:c r="H14"/>
       <x:c r="I14" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/reachy-mini-wireless.png</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/logitech-mk270.png</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>ROB-007</x:v>
+        <x:v>PER-001</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>Charger</x:v>
-      </x:c>
-      <x:c r="C15"/>
-      <x:c r="D15"/>
+        <x:v>Mouse</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Logitech</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>MK270</x:v>
+      </x:c>
       <x:c r="E15"/>
       <x:c r="F15" t="n">
         <x:v>1</x:v>
@@ -4944,18 +4942,22 @@
       </x:c>
       <x:c r="H15"/>
       <x:c r="I15" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/logitech-mk270.png</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>ROB-007</x:v>
+        <x:v>PER-001</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>USB Cable</x:v>
-      </x:c>
-      <x:c r="C16"/>
-      <x:c r="D16"/>
+        <x:v>USB receiver</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Logitech</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>MK270</x:v>
+      </x:c>
       <x:c r="E16"/>
       <x:c r="F16" t="n">
         <x:v>1</x:v>
@@ -4963,14 +4965,16 @@
       <x:c r="G16" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="H16"/>
+      <x:c r="H16" t="str">
+        <x:v>Nano receiver for this keyboard and mouse set</x:v>
+      </x:c>
       <x:c r="I16" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment-placeholder.svg</x:v>
+        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/logitech-mk270.png</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>PER-001</x:v>
+        <x:v>PER-002</x:v>
       </x:c>
       <x:c r="B17" t="str">
         <x:v>Keyboard</x:v>
@@ -4995,7 +4999,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>PER-001</x:v>
+        <x:v>PER-002</x:v>
       </x:c>
       <x:c r="B18" t="str">
         <x:v>Mouse</x:v>
@@ -5020,7 +5024,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>PER-001</x:v>
+        <x:v>PER-002</x:v>
       </x:c>
       <x:c r="B19" t="str">
         <x:v>USB receiver</x:v>
@@ -5047,7 +5051,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
-        <x:v>PER-002</x:v>
+        <x:v>PER-003</x:v>
       </x:c>
       <x:c r="B20" t="str">
         <x:v>Keyboard</x:v>
@@ -5072,7 +5076,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
-        <x:v>PER-002</x:v>
+        <x:v>PER-003</x:v>
       </x:c>
       <x:c r="B21" t="str">
         <x:v>Mouse</x:v>
@@ -5097,7 +5101,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
-        <x:v>PER-002</x:v>
+        <x:v>PER-003</x:v>
       </x:c>
       <x:c r="B22" t="str">
         <x:v>USB receiver</x:v>
@@ -5124,7 +5128,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
-        <x:v>PER-003</x:v>
+        <x:v>PER-004</x:v>
       </x:c>
       <x:c r="B23" t="str">
         <x:v>Keyboard</x:v>
@@ -5149,7 +5153,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
-        <x:v>PER-003</x:v>
+        <x:v>PER-004</x:v>
       </x:c>
       <x:c r="B24" t="str">
         <x:v>Mouse</x:v>
@@ -5174,7 +5178,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
-        <x:v>PER-003</x:v>
+        <x:v>PER-004</x:v>
       </x:c>
       <x:c r="B25" t="str">
         <x:v>USB receiver</x:v>
@@ -5201,7 +5205,7 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
-        <x:v>PER-004</x:v>
+        <x:v>PER-005</x:v>
       </x:c>
       <x:c r="B26" t="str">
         <x:v>Keyboard</x:v>
@@ -5226,7 +5230,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
-        <x:v>PER-004</x:v>
+        <x:v>PER-005</x:v>
       </x:c>
       <x:c r="B27" t="str">
         <x:v>Mouse</x:v>
@@ -5251,7 +5255,7 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
-        <x:v>PER-004</x:v>
+        <x:v>PER-005</x:v>
       </x:c>
       <x:c r="B28" t="str">
         <x:v>USB receiver</x:v>
@@ -5277,81 +5281,37 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" t="str">
-        <x:v>PER-005</x:v>
-      </x:c>
-      <x:c r="B29" t="str">
-        <x:v>Keyboard</x:v>
-      </x:c>
-      <x:c r="C29" t="str">
-        <x:v>Logitech</x:v>
-      </x:c>
-      <x:c r="D29" t="str">
-        <x:v>MK270</x:v>
-      </x:c>
+      <x:c r="A29"/>
+      <x:c r="B29"/>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
       <x:c r="E29"/>
-      <x:c r="F29" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G29" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
+      <x:c r="F29"/>
+      <x:c r="G29"/>
       <x:c r="H29"/>
-      <x:c r="I29" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/logitech-mk270.png</x:v>
-      </x:c>
+      <x:c r="I29"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" t="str">
-        <x:v>PER-005</x:v>
-      </x:c>
-      <x:c r="B30" t="str">
-        <x:v>Mouse</x:v>
-      </x:c>
-      <x:c r="C30" t="str">
-        <x:v>Logitech</x:v>
-      </x:c>
-      <x:c r="D30" t="str">
-        <x:v>MK270</x:v>
-      </x:c>
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
       <x:c r="E30"/>
-      <x:c r="F30" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G30" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
+      <x:c r="F30"/>
+      <x:c r="G30"/>
       <x:c r="H30"/>
-      <x:c r="I30" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/logitech-mk270.png</x:v>
-      </x:c>
+      <x:c r="I30"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" t="str">
-        <x:v>PER-005</x:v>
-      </x:c>
-      <x:c r="B31" t="str">
-        <x:v>USB receiver</x:v>
-      </x:c>
-      <x:c r="C31" t="str">
-        <x:v>Logitech</x:v>
-      </x:c>
-      <x:c r="D31" t="str">
-        <x:v>MK270</x:v>
-      </x:c>
+      <x:c r="A31"/>
+      <x:c r="B31"/>
+      <x:c r="C31"/>
+      <x:c r="D31"/>
       <x:c r="E31"/>
-      <x:c r="F31" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G31" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H31" t="str">
-        <x:v>Nano receiver for this keyboard and mouse set</x:v>
-      </x:c>
-      <x:c r="I31" t="str">
-        <x:v>https://pair-lab-imperial.github.io/nfc-inventory/assets/equipment/logitech-mk270.png</x:v>
-      </x:c>
+      <x:c r="F31"/>
+      <x:c r="G31"/>
+      <x:c r="H31"/>
+      <x:c r="I31"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -5364,7 +5324,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39a9becd9f514c35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4d75266a3e1472d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5487,7 +5447,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35ccca0549894800"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfadc1275e962498f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5661,7 +5621,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88b6b225f2844c98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f76eecd563043ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>